<commit_message>
Add 4 more leads and a community connector, found via targeted LinkedIn search
New leads: Katheryn Hunt (GROW Marketing Agency, confirmed 1-17 employees),
Adam Goyette (Growth Union), David Malevsky (Lynx Growth Agency), Alex Zlotko
(Forecastio) -- all sourced via site:linkedin.com/in and site:linkedin.com/posts
queries, which is the only LinkedIn surface reachable without login/scraping.
Also adds Mike Rizzo (MarketingOps.com / MO Pros) to Connectors -- he runs the
MO Pros community the outreach doc names as a target source.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -704,9 +704,181 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Katheryn Hunt</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>GROW Marketing Agency (St. Louis, MO)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/katherynhunt/</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small digital marketing agency (web design, digital marketing, branding). Confirmed small: 1-10 employees per Crunchbase, ~17 per ContactOut -- either way solidly inside the 5-50 band.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed small-agency founder wearing the ops hat -- one of the cleanest company-size confirmations in this batch.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Adam Goyette</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Growth Union (Chicago) -- boutique growth agency for early-stage B2B SaaS</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/adam-goyette/</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Ex-Help Scout / G2 growth marketing exec, now runs a small agency assembling senior marketers for early-stage B2B SaaS clients (Writer, RevenueHero, Recorded Future named as clients). Exact employee count unconfirmed but the agency's model (small senior team, no bench) implies well under 50.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Founder running a lean agency serving exactly the small-SaaS client base multiplayer targets; company size inferred from agency model, not directly confirmed -- worth a second look before approving.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>David Malevsky</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Lynx Growth Agency (Hallandale Beach, FL)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/david-malevsky/</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a boutique agency (patient acquisition for regenerative/integrative clinics) built around AI-driven marketing and automation. Employee count unconfirmed -- RocketReach shows only a handful of verified staff, consistent with a small shop.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Self-describes as 'resolving business challenges using AI' -- co-founder at a small, AI-forward agency is a strong qualitative fit even though the exact headcount isn't independently confirmed.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Alex Zlotko</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Forecastio (B2B sales forecasting for HubSpot)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alexzlotko/</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>17 years in B2B sales/CS, now CEO of Forecastio, a small SaaS company building sales forecasting tools. Publishes regularly on AI agents in RevOps specifically.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Small SaaS founder/CEO already writing publicly about AI agents in RevOps -- direct thematic overlap with multiplayer's pitch, though exact headcount at Forecastio is unconfirmed.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -720,7 +892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -867,9 +1039,52 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Mike Rizzo</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>MarketingOps.com / MO Pros</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mikedrizzo/</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Founded and runs MO Pros, the 4,000+ member marketing-ops community outreach-pipeline-context.md names directly as a target community. Certifies GTM Ops teams and runs the annual MOpza conference.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Not a cold-outreach target -- he IS the gatekeeper of the exact community your context doc lists as a source. Worth a warmer, separate approach (community partnership / sponsorship) rather than a first-touch DM template.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add 6 more leads and make profile links clickable in the sheet
New: Kristofer Wille, Donna Sluijter, John McArdle, Roberto Guerra,
Kristy Buige, Johnathan Wang -- all small RevOps/SaaS consultancy
founders/operators found via site:linkedin.com/in search, self-described
in ICP-matching language.

finder.py now writes the Profile/Post Link column as a real clickable
Excel hyperlink instead of plain URL text.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="001155CC"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -57,10 +61,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -428,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -505,7 +512,7 @@
           <t>PrecisionRevOps LLC</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/elizabeth-danowski-8b264513/</t>
         </is>
@@ -548,7 +555,7 @@
           <t>Lamande LLC (fractional RevOps for early/mid-stage SaaS); concurrent fractional roles at Rev, AgentSync, Ekho, OperateWise</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/jeremy-lamande/</t>
         </is>
@@ -591,7 +598,7 @@
           <t>Revenue Wizards</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/posts/harisodobasic_what-does-revops-do-revenue-operations-activity-7263475951290740736-3JwA</t>
         </is>
@@ -634,7 +641,7 @@
           <t>Independent — C-Suite advisor across SaaS/AI/startup clients</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/deepa--patel/</t>
         </is>
@@ -677,7 +684,7 @@
           <t>Independent — B2B SaaS clients (~$2M+ ARR)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/mariyavaleva-yourscalingpartner/</t>
         </is>
@@ -720,7 +727,7 @@
           <t>GROW Marketing Agency (St. Louis, MO)</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/katherynhunt/</t>
         </is>
@@ -763,7 +770,7 @@
           <t>Growth Union (Chicago) -- boutique growth agency for early-stage B2B SaaS</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/adam-goyette/</t>
         </is>
@@ -806,7 +813,7 @@
           <t>Lynx Growth Agency (Hallandale Beach, FL)</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/david-malevsky/</t>
         </is>
@@ -849,7 +856,7 @@
           <t>Forecastio (B2B sales forecasting for HubSpot)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/alexzlotko/</t>
         </is>
@@ -876,12 +883,287 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Kristofer Wille</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>RevOps Consultant &amp; Advisor</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- RevOpsVision (Berlin)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kriswille-revopsvision-revenue-operations-consultant-advisory/</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>10+ years in SalesOps/RevOps in Berlin's startup scene. Self-positions explicitly as helping 'C-Level Leaders &amp; Startups Supercharge Their Small RevOps Teams' -- his own tagline names the exact ICP.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>His public positioning IS the ICP description almost word-for-word (small RevOps teams at startups). Company size self-described, not independently verified.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Donna Sluijter</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Startup Operator -- RevOps &amp; Strategy</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Independent / embedded RevOps for startups</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/donnasluijter/</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Self-describes as a 'Startup Operator' bridging gaps and scaling teams in RevOps and strategy roles -- language that matches the ICP's 'founder wearing every hat' profile.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Title and self-description line up with the ICP almost exactly; specific current employer/headcount not independently confirmed.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>John McArdle</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sequoia Solutions -- RevOps/HubSpot consultancy for early-stage B2B tech</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/john-mcardle-m-s-71b58178/</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Founded a small consultancy that has worked with dozens of early-stage companies cleaning up CRM/HubSpot data and building GTM systems -- not the 'Sequoia' VC firm, a separate small boutique of the same name.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Founder-led small consultancy serving exactly the early-stage company band multiplayer targets.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Roberto Guerra</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Revenue Hub Latam -- RevOps + HubSpot for B2B companies in LATAM</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/robguerra/</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Runs a boutique RevOps/HubSpot consultancy for B2B companies across LATAM, publicly writing about pipeline, CRM, forecasting -- and AI.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Boutique consultancy founder already writing about AI in the RevOps workflow -- direct thematic and company-stage fit.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Kristy Buige</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Boutique RevOps consultancy -- B2B SaaS GTM systems</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kristybuige/</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Founded and leads a boutique RevOps consultancy enabling B2B SaaS companies to scale GTM systems, processes, and revenue performance.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small consultancy serving the same small-SaaS client base as several other rows in this sheet -- exact company name/size not independently confirmed beyond 'boutique.'</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Johnathan Wang</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>The SaaS Consultants -- fractional CMO / marketing agency for SaaS</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/johnathan-wang/</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Runs a small fractional-CMO agency for SaaS businesses and has personally built social-media-management software using Python/JavaScript and AI -- technical enough to be a strong early adopter.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder who is also hands-on technical/AI-building -- good combination of ICP fit and early-adopter likelihood.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -969,7 +1251,7 @@
           <t>Substack (independent) — background includes marketing ops leadership at Amazon</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://darrellalfonso.substack.com/</t>
         </is>
@@ -1012,7 +1294,7 @@
           <t>Substack (independent)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>https://jenbergren.substack.com/</t>
         </is>
@@ -1055,7 +1337,7 @@
           <t>MarketingOps.com / MO Pros</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/in/mikedrizzo/</t>
         </is>
@@ -1088,6 +1370,11 @@
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Draft Message column, generated from a fixed template per lead
finder.py now writes a personalized first-touch message for every lead,
built from a consistent template (operator/consultant/connector variant)
plus each row's one-line personal_detail, per Pipeline 2's personalization
style in outreach-pipeline-context.md. No auto-send exists (LinkedIn has
no pre-filled-message URL) -- workflow is click Profile Link, click
Message, paste Draft Message, edit, send.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -445,8 +445,9 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,10 +488,15 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Draft Message</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Date Found</t>
         </is>
@@ -532,8 +538,13 @@
           <t>Founder of a small (solo/very small) RevOps consulting shop -- exact ICP fit on company stage and role. Likely juggling multiple client workstreams solo, a strong proxy for the 'no shared visibility' pain.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Hey Elizabeth — saw you're running RevOps solo through PrecisionRevOps for multiple SaaS clients. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -575,8 +586,13 @@
           <t>Runs a small consulting practice AND sits inside multiple small SaaS teams concurrently (classic 5-50 person startup engagements) -- doubles as both a direct lead and a channel into several ICP companies at once.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jeremy — saw you're juggling fractional RevOps/CRO roles across Rev, AgentSync, Ekho, and OperateWise at once. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -618,8 +634,13 @@
           <t>Co-founder wearing the ops hat at a small consulting shop; his own public content (silos, alignment) lines up directly with the 'scattered, untracked work' pitch angle.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Hey Haris — saw your recent post on what RevOps actually does and removing GTM silos. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -661,8 +682,13 @@
           <t>Independent operator serving several small/startup clients in parallel -- same 'context lost across separate chats' problem multiplied across accounts rather than teammates.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Hey Deepa — saw you're advising several high-growth startups at once as a fractional RevOps/strategy leader. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -704,8 +730,13 @@
           <t>Ops-adjacent (finance) leader embedded in multiple small SaaS teams; weaker fit than the RevOps/MOps rows above but same team-size band and same fractional-across-many-small-teams dynamic -- worth a lower-priority pass.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Hey Mariya — saw you work as a fractional CFO across multiple early-stage B2B SaaS clients. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -747,8 +778,13 @@
           <t>Confirmed small-agency founder wearing the ops hat -- one of the cleanest company-size confirmations in this batch.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Hey Katheryn — saw you're running GROW Marketing Agency as a small, founder-led shop. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -790,8 +826,13 @@
           <t>Founder running a lean agency serving exactly the small-SaaS client base multiplayer targets; company size inferred from agency model, not directly confirmed -- worth a second look before approving.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Hey Adam — saw you've built a lean senior team at Growth Union for early-stage B2B SaaS clients like Writer and Recorded Future. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -833,8 +874,13 @@
           <t>Self-describes as 'resolving business challenges using AI' -- co-founder at a small, AI-forward agency is a strong qualitative fit even though the exact headcount isn't independently confirmed.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Hey David — saw you're building Lynx Growth Agency around AI-driven marketing and automation. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -876,8 +922,13 @@
           <t>Small SaaS founder/CEO already writing publicly about AI agents in RevOps -- direct thematic overlap with multiplayer's pitch, though exact headcount at Forecastio is unconfirmed.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Hey Alex — saw your writing on AI agents in RevOps as CEO of Forecastio. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -919,8 +970,13 @@
           <t>His public positioning IS the ICP description almost word-for-word (small RevOps teams at startups). Company size self-described, not independently verified.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Hey Kristofer — saw your tagline about helping startups supercharge their small RevOps teams. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -962,8 +1018,13 @@
           <t>Title and self-description line up with the ICP almost exactly; specific current employer/headcount not independently confirmed.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Hey Donna — saw your work bridging gaps and scaling teams as a startup RevOps operator. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -1005,8 +1066,13 @@
           <t>Founder-led small consultancy serving exactly the early-stage company band multiplayer targets.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Hey John — saw the dozens of early-stage companies you've helped clean up CRM/HubSpot data at Sequoia Solutions. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -1048,8 +1114,13 @@
           <t>Boutique consultancy founder already writing about AI in the RevOps workflow -- direct thematic and company-stage fit.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Hey Roberto — saw your posts on pipeline, forecasting, and AI at Revenue Hub Latam. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -1091,8 +1162,13 @@
           <t>Founder of a small consultancy serving the same small-SaaS client base as several other rows in this sheet -- exact company name/size not independently confirmed beyond 'boutique.'</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Hey Kristy — saw scaling GTM systems for B2B SaaS companies through your boutique RevOps consultancy. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -1134,8 +1210,13 @@
           <t>Small agency founder who is also hands-on technical/AI-building -- good combination of ICP fit and early-adopter likelihood.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Hey Johnathan — saw you built your own AI-powered social media tooling while running The SaaS Consultants. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -1143,7 +1224,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1174,7 +1255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1184,8 +1265,9 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1226,10 +1308,15 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Draft Message</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Date Found</t>
         </is>
@@ -1271,8 +1358,13 @@
           <t>Not a direct ICP lead -- flagged separately as a possible content/community distribution channel into the exact audience (marketing ops leads at small teams) rather than a cold-outreach target.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Hey Darrell — saw your newsletter on marketing ops team structure and career growth. I'm building multiplayer, a shared AI workspace for small ops teams — not pitching the community, just curious whether the 'everyone's using ChatGPT/Claude solo, zero shared visibility' problem is something you hear from members often. Open to a quick chat, and happy to share back whatever I learn.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -1314,8 +1406,13 @@
           <t>Same as Darrell Alfonso above -- a distribution/connector play into the ICP audience, not a direct 5-50 person company lead.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jen — saw your weekly newsletter for the marketing ops community. I'm building multiplayer, a shared AI workspace for small ops teams — not pitching the community, just curious whether the 'everyone's using ChatGPT/Claude solo, zero shared visibility' problem is something you hear from members often. Open to a quick chat, and happy to share back whatever I learn.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -1357,8 +1454,13 @@
           <t>Not a cold-outreach target -- he IS the gatekeeper of the exact community your context doc lists as a source. Worth a warmer, separate approach (community partnership / sponsorship) rather than a first-touch DM template.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Hey Mike — saw MO Pros hitting 4,000+ marketing/RevOps members. I'm building multiplayer, a shared AI workspace for small ops teams — not pitching the community, just curious whether the 'everyone's using ChatGPT/Claude solo, zero shared visibility' problem is something you hear from members often. Open to a quick chat, and happy to share back whatever I learn.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
@@ -1366,7 +1468,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add 15 more leads (30 total) from small agencies, HubSpot partners, chief-of-staff roles
Round 3 of LinkedIn public-page search: SEO/creative/content agency founders,
HubSpot partner agency operators, and two chief-of-staff hires at very
early-stage startups. Several rows flagged as single-source/lower-confidence
in match_reason -- worth a second look before approving those specifically.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1222,9 +1222,729 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Shaun Anderson</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>thisisagency.ai / hobo-web.co.uk -- forensic SEO agency</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/shaun-anderson-hobo/</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small forensic-SEO agency, also positions himself as an AI Marketing Engineer building agentic AI systems. Found via a single search pass, not cross-verified for exact headcount.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder already hands-on with agentic AI -- strong thematic fit; company size inferred from agency type, not confirmed.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Hey Shaun — saw you're building agentic AI systems as an AI Marketing Engineer while running thisisagency.ai. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Jackie Connors</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Digital Marketing Direction -- virtual HubSpot partner agency</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jackiebconnors/</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small virtual agency offering HubSpot/inbound training, consulting and content marketing. Size not independently confirmed beyond 'virtual agency' framing.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Founder-led small HubSpot partner shop -- same ops-tooling audience multiplayer is targeting.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jackie — saw you run Digital Marketing Direction as a virtual HubSpot partner agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Sam Anderson</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Chief Growth Officer / Founder</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Origin 63 -- small growth agency</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/samanderson41/</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Founder-level growth leader at a self-described small agency. Weaker verification than other rows -- single search snippet only.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Small growth-agency founder; include but treat as lower-confidence given only one source found.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Hey Sam — saw you're running Origin 63 as a small, results-focused growth agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Josh Harcus</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Revenue Growth &amp; Retention Lead</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hüify -- HubSpot partner agency</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/joshharcus/</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Works on revenue growth/retention at a HubSpot partner agency. Exact headcount at Hüify unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>HubSpot-partner-agency operator in the ops-tooling audience; company size inferred, not confirmed.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Hey Josh — saw your work on revenue growth and retention at Hüify, a HubSpot partner agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Alex Williams</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Independent HubSpot Consultant</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- solo HubSpot consulting practice</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/awoxford/</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Solo independent HubSpot implementation/strategy consultant -- a one-person shop, which is close to the purest form of the 'wearing every hat, no one to share tool context with' ICP signal.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Solo consultant -- exact company-stage fit by definition, though this is a one-person 'team' rather than 5-50 people; worth including as a different flavor of the same pain (no one to share context with at all).</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Hey Alex — saw you run your own solo HubSpot consulting practice. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Clwyd Probert</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder, AI Consultant</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Whitehat (UK) -- AI consulting</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/in/clwyd-probert</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>CEO/Founder and AI consultant; company size and exact scope of Whitehat not independently confirmed -- single search snippet only.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Directly in the AI-adoption-for-small-business space -- strong thematic fit, weaker company-size confirmation.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Hey Clwyd — saw you work as an AI consultant at Whitehat, helping businesses adopt AI. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Clara Ma</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff (Employee #3)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Kairos -- very early-stage startup</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/clarama/</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff at a very early-stage startup (self-described as employee #3) -- partners with founders through the hardest parts of scaling. About as small/early as the ICP gets.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Employee #3 at an early-stage startup wearing the ops/chief-of-staff hat -- textbook ICP fit on company stage.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Hey Clara — saw you're employee #3 and Chief of Staff at Kairos. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Josephine Conneely</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff -- GTM, Operations, AI</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed (UK-based startup)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/in/josephineconneely</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff with GTM/Operations/AI explicitly in her title -- current employer name and headcount not independently confirmed.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Title puts AI and ops in the same remit -- strong thematic fit; company-size confirmation weaker than other rows.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Hey Josephine — saw your Chief of Staff role spanning GTM, Operations, and AI. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Riddhi Sharma</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Thought In A Dot -- content marketing agency</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sharmariddhi/</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>14+ years in leadership/brand content strategy, now founder/CEO of a content marketing agency. Employee count unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder in the marketing-ops-adjacent content space.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Hey Riddhi — saw you're running Thought In A Dot as a content marketing agency and brand strategist. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>John Liska</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Creative Engine (Austin, TX) -- branding &amp; digital marketing agency</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/john-liska-594a52193/</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small branding/digital marketing agency in Austin. Employee count unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder -- fits the company-stage band, size inferred not confirmed.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Hey John — saw you founded Creative Engine, a branding and digital marketing agency in Austin. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Ajay G.</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>MAWD Agency -- Google Ads/SEO/websites for small businesses</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ajayg514/</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small AI-forward performance-marketing agency serving small-business clients.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder in the exact small-business-serving segment; last-name not public in the source, listed as found.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Hey Ajay — saw you run MAWD Agency managing Google Ads, SEO, and websites for small businesses. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Raj Goodman Anand</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Goodman Lantern -- B2B content marketing agency</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rajanand/</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a B2B content marketing agency serving clients across several continents -- distributed small team model, not independently headcount-confirmed.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Founder wearing the ops/marketing hat; 'across five continents' framing suggests a distributed small team rather than a large single office, but worth double-checking size before approving.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Hey Raj — saw you're running Goodman Lantern, a B2B content marketing agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Laney M. Silverman</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>The Design Boutique, Inc.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/thedesignboutique/</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a self-described boutique design agency, explicitly positioned around small-team speed/agility.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly 'boutique' self-positioning -- good qualitative company-size signal even without a hard headcount number.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Hey Laney — saw you run The Design Boutique and pride yourselves on being able to pivot quickly as a small shop. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Thomas Kranzle</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Founder, Director</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Venture Visuals (Seattle) -- creative agency</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/thomaskranzle/</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Founder/Director of a small creative agency in Seattle. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder -- company-stage fit inferred from agency type.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Hey Thomas — saw you founded Venture Visuals, a creative agency in Seattle. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Santosh Kushwaha</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Visual Best -- AI Creative Production Agency</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/in/santosh-kushwaha-explorer</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small, explicitly AI-native creative production agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>AI-native agency founder -- strong thematic fit, company size inferred not confirmed.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Hey Santosh — saw you're running Visual Best, an AI creative production agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1244,6 +1964,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 14 more leads (43 total): e-commerce, dev shops, recruiting, bookkeeping
Round 4: small Shopify/ecommerce agencies, AI-native software consultancies,
solo AI consultants, one YC-backed early-stage founder, performance marketing
agencies (incl. one specializing in B2B SaaS ads), boutique recruiting
agencies, and a few finance-ops-adjacent bookkeeping practices for
diversification. All sourced via site:linkedin.com/in search.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1942,9 +1942,633 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>David Simões</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Sounds Good Agency -- Shopify Plus partner (CEE region)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>https://cz.linkedin.com/in/davidjsimoes/en</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a Shopify Plus agency serving DTC/B2B/Retail brands, self-describes as having an 'AI-first business mindset.' Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder explicitly framing the business around AI-first thinking -- strong thematic fit.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Hey David — saw you describe your business as having an AI-first mindset while running Sounds Good Agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Mark Kennaley</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>SoftwareFactory.ai -- AI-native software engineering consultancy</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/markkennaley/</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small AI-native software engineering consultancy. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Small AI-forward software consultancy founder -- exactly the kind of technical early adopter this product needs.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Hey Mark — saw you're a pioneer in AI-native software engineering as founder of SoftwareFactory.ai. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Philip Ledgerwood</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>AI Consultant / Software Developer</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- solo AI consulting practice</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/phil-ledgerwood/</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Solo independent consultant helping companies adopt AI securely. One-person practice -- same 'no one to share context with' signal as other solo consultants in this sheet.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Solo AI consultant -- direct thematic fit and purest form of the company-stage signal.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Hey Philip — saw you help companies use AI securely and purposefully as an independent consultant. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Dylan Kinder</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Independent AI Consultant</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- installs AI systems into service businesses</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/dylankinder/</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Solo consultant helping small service businesses adopt AI tooling. Weaker verification -- single search snippet only.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Solo AI-adoption consultant serving small businesses -- direct thematic fit, lower-confidence single-source finding.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Hey Dylan — saw you install AI systems into service businesses as an independent consultant. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Alex Marantelos</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder / CEO</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Intryc (Y Combinator S24)</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alexmarantelos/</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a YC S24-batch startup -- confirmed very-early-stage by accelerator batch, though exact current headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage (accelerator batch is public record) even without a hard headcount number.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Hey Alex — saw you're co-founder/CEO of Intryc, a Y Combinator S24 startup. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Arham Khan</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Pixated -- performance marketing agency (paid social/search)</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/in/arhamkhan</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small performance marketing agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder -- company-stage fit inferred from agency type.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Hey Arham — saw you founded Pixated, a performance marketing agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Alex Brown</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Tierra -- performance marketing agency for DTC ecommerce</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alex-brown-tierra/</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small performance marketing agency for DTC ecommerce brands. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder -- company-stage fit inferred from agency type.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Hey Alex — saw you're scaling DTC ecommerce brands through Tierra. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Oles Dziub</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Hey Digital -- SaaS performance marketing &amp; creative agency</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/oles-dziub-b2b-saas-paid-ads-expert/</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a small agency specializing in paid ads for B2B SaaS companies -- serves exactly multiplayer's target client base.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Agency founder specializing in the B2B SaaS vertical multiplayer targets -- strong client-overlap fit.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Hey Oles — saw you're running Hey Digital, a performance marketing agency focused specifically on B2B SaaS. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Beckie Blackburn-Cooper</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Boutique recruiting agency</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/beckie-blackburn-cooper-bri/</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small, self-described boutique recruiting agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly 'boutique' self-positioning -- good qualitative size signal; different vertical (recruiting) than most of this sheet, useful diversification.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Hey Beckie — saw you run a boutique recruiting agency with a niche sector focus. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Katie Matthews</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>CollabRecruit -- small recruiting agency</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kmtalentfinder/</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small recruiting agency, writes publicly about technology's role in staffing. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder already thinking publicly about tech's role in her business -- good adoption-readiness signal.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Hey Katie — saw your writing on balancing technology and human connection in recruiting at CollabRecruit. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Becky Kuntz</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>BK's Bookkeeping</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/becky-kuntz/</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small virtual bookkeeping practice serving small-business clients. Finance-ops-adjacent, similar band to Mariya Valeva elsewhere in this sheet.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Small finance-ops shop founder -- weaker fit than marketing/RevOps rows but same company-stage band and same 'wearing every hat' pain.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Hey Becky — saw you help small business owners get time back through BK's Bookkeeping. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Tom Wells</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Business Development</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Wells Virtual Bookkeeping, LLC</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tom-wells-rad60/</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Small virtual bookkeeping practice; actively participates in an AI Mastermind group -- already engaged with AI adoption specifically.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Small ops-adjacent shop already active in an AI-adoption community -- good readiness signal despite being outside core marketing/RevOps.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Hey Tom — saw you're part of an AI Mastermind group applying tech-forward solutions to bookkeeping. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Jennifer Perez-Fong</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Bookkeeping Done Right</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jennifer-perez-fong-cpa/</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>CEO/founder of a small accounting practice serving SMBs, founded 2013. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Small finance-ops shop founder -- same lower-priority band as other bookkeeping rows in this sheet.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jennifer — saw you founded Bookkeeping Done Right to serve small and medium businesses in South Florida. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1979,6 +2603,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 15 more leads (58 total): PR, design/creative, early-stage co-founders, PPC
Round 5: small PR/comms agencies, design/creative agency founders (several
explicitly self-describing as 'small team'), early-stage startup co-founders
wearing the ops hat directly, PPC agencies specializing in B2B SaaS clients,
and AI-forward video/media production founders.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2566,9 +2566,729 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Parry Headrick</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Crackle PR -- B2B tech PR agency (Boston)</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/parryheadrick/</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small B2B tech PR agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>B2B-tech-focused small agency founder -- adjacent vertical (PR) serving the same kind of small SaaS/tech clients.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Hey Parry — saw you're leading a team of senior PR leaders at Crackle PR. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Carin Warner</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Warner Communications -- PR &amp; comms strategy</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carinwarner/</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a small PR/comms firm, publishes on AI strategy in communications specifically. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Small agency co-founder already writing about AI strategy in her own field -- strong thematic fit.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Hey Carin — saw your writing on AI strategy in communications. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Erika Torres</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>85th &amp; Park Inc. -- creative marketing &amp; communications agency</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/erika-torres85/</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small creative marketing/communications agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder -- company-stage fit inferred from agency type.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Hey Erika — saw you're running 85th &amp; Park, a culture-driven creative marketing and comms agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Sam Poutakidis</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>New AI Automation Agency</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sampoutakidis/</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a brand-new AI automation agency. Very early-stage by definition; single search snippet only.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Newest-stage AI-native agency founder in this sheet -- strong thematic fit, lower-confidence single-source finding.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Hey Sam — saw you just founded a new AI automation agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>M Kazemi</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Web design agency (Issaquah, WA)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/m-kazemi-098880242/</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small web design agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder -- company-stage fit inferred from agency type.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Hey M — saw you're running your own web design agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Michael Lieu</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Boldly -- design agency (London)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michael-lieu-77746972/</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of an award-winning design agency explicitly described as a small team. Good qualitative size signal.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly 'small team' self-positioning -- solid company-size signal without a hard headcount number.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Hey Michael — saw you're running Boldly with a small team of creative minds. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Kristen Ransom</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>CTO &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>IncluDe Web Design and Development Agency</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kristen-m-ransom/</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>CTO/Founder of a small web design/dev agency, publicly interested in AI adoption for the field. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Technical founder already thinking about AI adoption -- good early-adopter signal.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Hey Kristen — saw your interest in AI adoption for web design and development. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Stefen Phelps</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Kelp Creative Agency</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/stefenphelps/</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Software engineer and co-founder of a small creative agency. Headcount unconfirmed -- single search snippet only.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Technical co-founder at a small creative agency -- good blend of ICP fit and technical early-adopter likelihood.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Hey Stefen — saw you co-founded Kelp Creative Agency. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Dean Swennumson</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder, Head of Operations</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Superstate</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/dean-swennumson-075798125/</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder wearing the Head of Operations hat at an early-stage startup. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Textbook 'founder wearing the ops hat' ICP fit; company size inferred from co-founder/early-stage framing, not confirmed.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Hey Dean — saw you're co-founder and Head of Operations at Superstate. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Leah Bolden</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; Head of Operations</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>See Jane Drill</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/leah-bolden-24419314</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/Head of Operations at a small DIY-resource startup. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Founder wearing the ops hat at an early-stage company -- solid ICP fit by role and company stage.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Hey Leah — saw you're co-founder and Head of Operations at See Jane Drill. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Michael McCormack</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; COO</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>10X ERP</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michael-mccormack-10xerp/</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/COO of a small startup, explicitly noted as acting as the de-facto Operations Manager -- wearing multiple hats.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder explicitly wearing both COO and hands-on ops-manager hats -- strong 'founder wearing every hat' ICP fit.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Hey Michael — saw you're co-founder and de-facto Operations Manager at 10X ERP. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Pavels Mordvicevs</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Camel Digital -- PPC agency for B2B SaaS</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/pavels-mordvicevs-2aaa4666/</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small PPC agency explicitly targeting B2B SaaS founders -- serves exactly multiplayer's target client base.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Agency founder specializing in the B2B SaaS vertical multiplayer targets -- strong client-overlap fit, same pattern as Oles Dziub.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Hey Pavels — saw you're targeting B2B SaaS founders specifically through Camel Digital. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Aaron Arnold</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>FeatherDot Media Group LLC -- video production/growth</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/fdmg/</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small video production/growth agency, explicitly positions AI repurposing as part of the offering.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>AI-forward small agency founder -- direct thematic fit.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Hey Aaron — saw your work helping brands scale with strategic video content and AI repurposing. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Evan Cassidy</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Boomin' Brands Media</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/evanbcassidy/</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small creative media agency, already using AI content tools in production. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder already hands-on with AI production tools -- good early-adopter signal.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Hey Evan — saw you're using AI tools like Heygen and Freepik at Boomin' Brands Media. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Yash Arora</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Founder / Producer</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Lemonade Creatives</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/yasharora16/</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Founder/producer of a small creative production studio incorporating AI-led production. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder already building AI into the production pipeline -- direct thematic fit.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Hey Yash — saw your AI-led creative production work at Lemonade Creatives. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2616,6 +3336,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 20 more leads (78 total), including 10 YC-batch co-founders
Round 6: 10 Y Combinator (S24/S25/W25) co-founders -- accelerator batch is
public record, so company stage is independently confirmed rather than
self-described, several building AI-native products themselves. Plus small
consultancy/agency founders in localization, design, customer success, legal
tech, and influencer marketing -- verticals not yet represented in this sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3286,9 +3286,969 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Paul Dietrich</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CPO</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Spherecast (Y Combinator S24)</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/pauldietrich98/</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CPO of a YC S24-batch startup -- accelerator batch is public record, confirming very-early company stage.</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage; technical co-founder role suggests strong early-adopter fit.</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Hey Paul — saw you're co-founder and CPO of Spherecast, a YC S24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Avi Konduru</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Shor (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/avi-konduru-54b3a6bb/</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage, textbook ICP by definition.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Hey Avi — saw you're co-founder of Shor, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Dhruv Roongta</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>slashy.com (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/dhruv-roongta-421a7b214/</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Hey Dhruv — saw you're co-founder of slashy.com, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Michael Kim</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>AgentMail (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michaelhyunkim/</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch startup building AI-agent-related infrastructure -- confirmed very-early stage and directly AI-native.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder in the AI-agent space itself -- strong thematic AND company-stage fit.</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Hey Michael — saw you're co-founder of AgentMail, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Ishaan Sehgal</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Omnara (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ishaan-sehgal/</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Hey Ishaan — saw you're co-founder of Omnara, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Raj Lad</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Infinite (Y Combinator W25)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/rajlad/</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W25-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Hey Raj — saw you're co-founder of Infinite, a YC W25 company, previously at Sardine. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Kushal Mohta</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Optifye.ai (Y Combinator W25)</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kushal-mohta-6926931b4/</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W25-batch AI startup -- confirmed very-early stage and directly AI-native.</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage AI founder -- strong thematic AND company-stage fit.</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Hey Kushal — saw you're co-founder of Optifye.ai, a YC W25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Nand Vinchhi</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Axal (Y Combinator W25)</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nandvinchhi/</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W25-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Hey Nand — saw you're co-founder of Axal, a YC W25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>William Barthell</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Janet AI (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/william-barthell/</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch AI startup -- confirmed very-early stage and directly AI-native.</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage AI founder -- strong thematic AND company-stage fit.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Hey William — saw you're co-founder of Janet AI, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Aditya Iyengar</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Candor (Y Combinator W25)</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/aditya-v-iyengar/</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W25-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Hey Aditya — saw you're co-founder of Candor, a YC W25 company focused on insider-risk. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Adam Wooten</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Taia -- translation workflow platform / AI consultant</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/adamwooten/</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Translation-tech/AI consultant and founder of a small workflow platform. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Small AI-native tooling founder -- direct thematic fit, different vertical (localization) for diversification.</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Hey Adam — saw you built Taia, a workflow system addressing friction in translation processes. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Ebru Yildirim</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Ollang -- localization</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ebru-yildirim-ollang/</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small localization company with two decades of enterprise localization experience, publicly skeptical of AI-solves-everything narratives -- a thoughtful, engaged voice.</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder actively engaging with AI's real limits in her field -- a more skeptical but still relevant prospect.</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Hey Ebru — saw your take that AI translating doesn't mean localization is solved. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Adriana Biarnes Garcia</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Libre Design Studio -- design studio for founders/startups</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/adriana-biarnes-garcia/</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small design studio explicitly positioned to serve founders/startups. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Small studio founder serving the exact startup client base multiplayer targets.</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Hey Adriana — saw you run Libre Design Studio specifically for founders and startups. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Atiqur Rahaman</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Design Monks</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/atiq31416/</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small design agency. Headcount unconfirmed -- single search snippet only.</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder -- company-stage fit inferred from agency type, lower-confidence single-source finding.</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Hey Atiqur — saw you founded Design Monks. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Crystal J. Morgan</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Fractional Customer Success Consultant</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- serves SaaS founders and CS teams</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/crystaljmorgan/</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Fractional Customer Success consultant serving multiple small SaaS clients at once -- same fractional-across-many-teams pattern as other consultant rows in this sheet.</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CS consultant across small SaaS clients -- ops-adjacent vertical (customer success) not yet represented in this sheet.</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Hey Crystal — saw you help SaaS founders and CS teams with customer success operations as a fractional consultant. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Thomas Christensen</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Revora Consultants -- Customer Success consulting for B2B SaaS</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/thomas-christensen-0814a39/</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small CS consultancy for B2B SaaS companies. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Small CS consultancy founder serving the exact small-SaaS client base multiplayer targets.</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Hey Thomas — saw you help B2B SaaS companies turn Customer Success into measurable revenue at Revora Consultants. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Peter Varga</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Lafluence &amp; Trendin -- AI-native OS for influencer agencies</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/petervarga1/</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Ex-Google, founder of two small companies including an explicitly AI-native product for influencer agencies. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>AI-native small-company founder -- direct thematic fit.</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Hey Peter — saw you're building Trendin, an AI-native operating system for influencer agencies. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Jamiu Akanbi</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Hidden Gems -- creator-led growth for B2B AI &amp; SaaS companies</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jamiu-akanbi/</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small agency specializing in B2B AI/SaaS client growth -- serves exactly multiplayer's target client base.</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Agency founder specializing in the B2B AI/SaaS vertical multiplayer targets -- strong client-overlap fit.</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jamiu — saw you're running Hidden Gems, focused on creator-led growth specifically for B2B AI &amp; SaaS companies. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Krishna Kammili</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>LegalConnect -- AI-assisted legal documents for SMEs</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/krishnakammili/</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small legal-tech company already combining AI drafting with human review. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>AI-native small-company founder in an underrepresented vertical (legal tech) -- direct thematic fit, good diversification.</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Hey Krishna — saw you built LegalConnect to deliver AI-drafted, solicitor-reviewed legal documents for SMEs. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Jay Pietig</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Founding Partner</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Startup Legal Group, LLC (Kansas City)</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jay-pietig-startuplegalgroup/</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Founding partner of a small legal practice explicitly serving startup clients. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Small legal practice founder serving the exact startup client base multiplayer targets -- underrepresented vertical for diversification.</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jay — saw you run Startup Legal Group, serving startup clients directly. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3351,6 +4311,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 19 more leads (97 total): more YC/Techstars co-founders + new verticals
Round 7: 10 more accelerator-backed early-stage co-founders (YC F24/W24,
Techstars), several explicitly AI-native small companies whose own mission
overlaps with multiplayer's, and small-agency founders in market research,
architecture/design, and MSP verticals for continued diversification.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4246,9 +4246,921 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Chris Pisarski</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Crustdata (Y Combinator F24)</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/chris-pisarski/</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC F24-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Hey Chris — saw you're co-founder of Crustdata, a YC F24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Manmohit Grewal</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Crustdata (Y Combinator F24)</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/manmohitgrewal/</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC F24-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Hey Manmohit — saw you're co-founder of Crustdata, a YC F24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Shawn Shivdat</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Penciled (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/shawn-shivdat/</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a YC W24-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Hey Shawn — saw you're co-founder and CEO of Penciled, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Sarah Hamer</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder / COO</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>RetailReady (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sarah-hamer/</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/COO of a YC W24-batch startup -- confirmed very-early stage, and she's the one directly wearing the ops hat.</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage COO -- exact 'founder wearing the ops hat' ICP fit with confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Hey Sarah — saw you're co-founder and COO of RetailReady, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Chris Aeberli</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Sonia (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/chris-aeberli/</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W24-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Hey Chris — saw you're co-founder of Sonia, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>William Wang</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Centralize (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/williamwang77/</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W24-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Hey William — saw you're co-founder of Centralize, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Andy Li</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Respan (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/hanheli/</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a YC W24-batch startup -- confirmed very-early stage by accelerator batch.</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Hey Andy — saw you're co-founder and CEO of Respan, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Givi Beridze</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>KLIPY (Techstars-backed)</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/giviberidze/</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a Techstars-backed early-stage startup -- confirmed very-early stage by accelerator affiliation.</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Accelerator-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Hey Givi — saw you're co-founder and CEO of KLIPY, a Techstars-backed company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Karla Valdivieso</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Shappi (Techstars-backed)</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kvaldivieso/</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a Techstars-backed early-stage startup -- confirmed very-early stage by accelerator affiliation.</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Accelerator-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Hey Karla — saw you're co-founder and CEO of Shappi, a Techstars-backed company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Harry Dixon</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Co-Founder</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Building mate -- AI growth teammate for small businesses</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/harryjdixon1/</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of an early-stage startup building an AI teammate product for small businesses -- directly AI-native and thematically adjacent.</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Early-stage AI-native founder building a directly adjacent product category -- strong thematic fit.</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Hey Harry — saw you're building 'mate,' an AI growth teammate for small businesses. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Mihai Iancu</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>MspCoreX -- AI-first platform for Managed Service Providers</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mihai-iancu-2605681a/</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small AI-first platform for MSPs -- directly AI-native, unifying-tools angle close to multiplayer's own pitch.</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>AI-native small-company founder building a product with a very similar 'unify fragmented tools' thesis.</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Hey Mihai — saw you're building MspCoreX to replace fragmented MSP tool stacks with one intelligent core. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Michelle McCulloch</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Real Marketing Muscle -- helps small/mid-sized agencies grow</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michelle-mcculloch-616b953/</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small consultancy explicitly focused on helping other small agencies grow -- both an ICP member and a possible channel into other small agencies.</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Small consultancy founder whose own client base is other small agencies -- potential dual lead/channel value.</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Hey Michelle — saw your mission of helping small and mid-sized agencies grow through Real Marketing Muscle. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Nahme Chokeir</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Research Connections, Inc. -- market research consulting</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nchokeir/</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small market research consultancy. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder in an underrepresented vertical (market research) for diversification.</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Hey Nahme — saw you're running Research Connections, a market research consulting and field management company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Jake Wujastyk</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>JakeWu Market Research</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jakewujastyk/</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Solo/very-small market research founder. Headcount unconfirmed -- single search snippet only.</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Solo-founder small shop -- purest form of the company-stage signal, lower-confidence single source.</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jake — saw you run JakeWu Market Research, a small solo-founder shop. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Moritz Schmidt</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>GEMESYS -- deeptech startup, confirmed under 10 people</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/schmidtmo/</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a deeptech startup explicitly described as under 10 people -- rare, directly confirmed headcount.</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>One of the few rows with an explicitly confirmed sub-10-person headcount -- very high-confidence ICP fit.</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Hey Moritz — saw you're co-founder of GEMESYS, a deeptech company with under 10 people. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Jenna Gaidusek</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>AI for Interior Designers -- educational platform</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jenna-gaidusek-33175a26/</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CEO of a small AI-education platform for a specific creative vertical (interior design). Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>AI-adoption-focused small-company founder in a new vertical (interior design) -- direct thematic fit.</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jenna — saw you founded an education platform teaching interior designers to use AI. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Nina Grondin</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Partner &amp; Co-Founder</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Curioso -- design/architecture studio collective</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nina-grondin/</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a small multidisciplinary design/architecture studio. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Small studio co-founder in an underrepresented vertical (architecture/design) for diversification.</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Hey Nina — saw you co-founded Curioso, an assemblage of designers, architects, and business-minded creatives. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Snehadeep Das</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; Chief Designer</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Studio ORCHIVIZ -- AI-driven architectural visualization</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/snehadeep-das-81203b16b/</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Founder/Chief Designer of a small AI-driven architectural visualization studio. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>AI-native small studio founder -- direct thematic fit, underrepresented vertical.</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Hey Snehadeep — saw you use AI-driven design tools as founder of Studio ORCHIVIZ. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Austin Richard</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>digital3 AI -- AI accessibility for entrepreneurs and small businesses</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/digital3ai/</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a small company focused on AI accessibility for small businesses -- directly aligned mission.</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>AI-native small-company co-founder whose own mission overlaps directly with multiplayer's target audience.</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Hey Austin — saw you're making AI accessible and practical for entrepreneurs and small business owners at digital3 AI. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4331,6 +5243,25 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId97"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 11 more leads (108 total): older YC batch + brand/content agencies
Round 8: 4 YC W23-batch founders (flagged with a caveat -- that batch is
~3 years old now, so current headcount needs re-verification before
approving, unlike the more recent S25/W25/F24 batches added earlier), plus
small AI-native content/brand-voice agencies and brand-strategy consultancies
serving early-stage startups. Dropped two candidates (Shandel, Pushkar Raj)
where the only profile URL found was actually someone else's -- excluded
rather than risk misattributing an identity.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J98"/>
+  <dimension ref="A1:J109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5158,9 +5158,537 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Akeem Williams</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Thread (Y Combinator W23)</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/akeem-k-williams/</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W23-batch startup. CAVEAT: this batch is ~3 years old as of now -- company may have grown well past the 5-50 band since the accelerator batch, worth re-checking current headcount before approving.</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed founder, but older batch than the other YC rows in this sheet -- lower confidence on current company size specifically.</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Hey Akeem — saw you're co-founder of Thread, a YC W23 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Ty Sharp</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>inBuild (Y Combinator W23)</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ty-sharp/</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a YC W23-batch startup. CAVEAT: batch is ~3 years old, current headcount may exceed the 5-50 band -- re-verify before approving.</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed founder, older batch -- lower confidence on current size.</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Hey Ty — saw you're co-founder and CEO of inBuild, a YC W23 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Vlad Matsiiako</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Infisical (Y Combinator W23)</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/vmatsiiako/</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W23-batch developer-tools startup. CAVEAT: batch is ~3 years old, current headcount may exceed the 5-50 band.</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed founder in dev tooling, older batch -- lower confidence on current size, still worth a look given the technical audience fit.</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>Hey Vlad — saw you're co-founder of Infisical, a YC W23 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Neel Balar</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Clueso -- AI video creation (Y Combinator W23)</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/neelbalar7/</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W23-batch AI startup. CAVEAT: batch is ~3 years old, current headcount may exceed the 5-50 band.</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>AI-native founder, older YC batch -- lower confidence on current size but strong thematic fit.</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Hey Neel — saw you're co-founder of Clueso, an AI video creation company from YC W23. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Yael Chen Zion</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Digital -- brand voice/content agency</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/yaelchenzion/</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small content/brand-voice agency, already building custom AI agents into the workflow -- directly AI-native.</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder already building bespoke AI agents -- strong thematic fit and technical sophistication.</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Hey Yael — saw you built an AI agent trained on multiple brand voices and content formats at Ashley Digital. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr"/>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Ai Jane L.</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Common AI -- AI/no-code accessibility for small businesses</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/aijane-common-ai/</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small company focused on AI accessibility for small businesses -- directly aligned mission with multiplayer's audience.</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>AI-native founder whose own mission is helping small businesses use AI -- direct thematic fit.</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Hey Ai — saw you're democratizing access to AI and no-code tools for individuals and small businesses through Common AI. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Vanhishikha Bhargava</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Contensify -- SEO/content for B2B SaaS</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>https://ae.linkedin.com/in/vanhishikhab</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small content/SEO agency specializing in B2B SaaS clients across martech, AI, HRtech, CRM and devtools.</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Agency founder specializing in the exact B2B SaaS vertical multiplayer targets -- strong client-overlap fit.</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Hey Vanhishikha — saw you've partnered with 100+ B2B SaaS companies on SEO and content through Contensify. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr"/>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Sourav Ganguly</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Branded Minds -- brand strategy for early-stage startups</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sourav-ganguly-3697904/</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small brand strategy agency serving early-stage startups. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder serving the exact early-stage startup client base multiplayer targets.</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Hey Sourav — saw you focus on brand strategy specifically for early-stage startups at Branded Minds. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Ulli Appelbaum</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; CSO</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>First The Trousers -- brand strategy and positioning consultancy</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ulliappelbaum/</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Founder/CSO of a small brand strategy consultancy. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Solo/small consultancy founder -- fits the consultant pattern in this sheet.</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Hey Ulli — saw you run First The Trousers as a brand strategy and positioning consultancy. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr"/>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Lance Mald</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>BrandChef.ai</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/lancemald/</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small, explicitly AI-named branding tool/agency. Headcount unconfirmed -- single search snippet only.</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>AI-native small-company founder -- direct thematic fit, lower-confidence single-source finding.</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Hey Lance — saw you're building BrandChef.ai. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Branden Lower</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Build -- branding agency</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/branden-lower-634b1b139/</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small branding agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder -- company-stage fit inferred from agency type.</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Hey Branden — saw you founded Build, a branding agency built around practical design. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr"/>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5262,6 +5790,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 20 more leads (128 total): 8 more YC S25 founders + HR/BI/SEO consultants
Round 9: 8 YC S25-batch co-founders including two with explicitly confirmed
headcounts (Pingo: team of 3; Munify: 20 people at $20M ARR -- among the
highest-confidence company-size matches in this sheet). Plus People
Ops/HR consultants serving startups and small agencies, B2B SaaS SEO/AI-search
consultants (one who just hired employee #1), BI consultants, and B2B podcast
agencies already engaging with AI in production.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J109"/>
+  <dimension ref="A1:J129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5686,9 +5686,969 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Morrie Schonfeld</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Pingo (Y Combinator S25) -- team of 3</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/morrie-schonfeld-1628002b1/</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch startup, confirmed team size of 3 -- as small and confirmed as this sheet gets.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed 3-person team -- extremely high-confidence ICP fit on company stage.</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Hey Morrie — saw you're co-founder of Pingo, a YC S25 company with a team of just 3 people. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Gurveer Singh</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Certus AI (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/gurveer-singh29/</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a YC S25-batch AI startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage AI founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Hey Gurveer — saw you're co-founder and CEO of Certus AI, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Alex Avnit</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Paloma -- AI-native CRM (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alex-avnit-222b3611a/</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch AI-native CRM startup -- confirmed very-early stage, ex-Deel/Revolut background.</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage AI founder -- confirmed company stage and directly AI-native product.</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Hey Alex — saw you're co-founder of Paloma, an AI-native CRM from YC S25. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Khalid A.</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Munify (Y Combinator S25) -- 20 people, $20M ARR</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/khalidashmawy/</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a YC S25-batch startup with an explicitly confirmed 20-person team -- rare, directly confirmed headcount right in the ICP's sweet spot.</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly confirmed 20-person team -- one of the highest-confidence company-size matches in this sheet.</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>Hey Khalid — saw you've grown Munify to $20M ARR with a team of just 20 people. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr"/>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Arjun Talati</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Knowlify (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/arjun-talati/</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Hey Arjun — saw you're co-founder of Knowlify, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Nazli Danis</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Paloma -- AI-native CRM (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nazlidanis/</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch AI-native CRM startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage AI founder -- confirmed company stage; second co-founder at Paloma alongside Alex Avnit, both worth reaching independently.</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>Hey Nazli — saw you're co-founder of Paloma, an AI-native CRM from YC S25. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr"/>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Neha Suresh</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Procindex (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nehasuresh1904/</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>Hey Neha — saw you're co-founder of Procindex, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>John Yeo</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Autumn (Y Combinator S25)</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/in/johnyeocx</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC S25-batch startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>Hey John — saw you're co-founder of Autumn, a YC S25 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr"/>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Susan Sarit</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Empower and Cultivate -- People Ops &amp; Systems consulting</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/susan-sarit/</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small People Ops consultancy explicitly supporting small business owners and founders.</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>Consultant serving the exact small-founder audience multiplayer targets, in an underrepresented vertical (people ops).</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Hey Susan — saw you help founders build self-sufficient teams as a People Ops &amp; Systems consultant. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Heidi R. Haskins</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Elevated Prana People Ops Consulting</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/heidiparks/</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small People Ops consultancy focused on startups and tech companies specifically.</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>Consultant explicitly serving the startup/tech audience multiplayer targets.</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>Hey Heidi — saw you focus on People Ops/HR solutions specifically for startups and tech companies. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr"/>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Michelle Dicks</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Quantum People Ops</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michelle-dicks-3872a791/</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>Owner of a small People Ops consultancy providing scalable HR systems for growing teams.</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>Consultant in the people-ops vertical serving growing small teams.</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>Hey Michelle — saw you provide scalable HR systems for growing teams through Quantum People Ops. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr"/>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Danielle Laurent</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Founder's HR Lab</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/danielle-laurent/</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small HR consultancy explicitly focused on building systems for small businesses and agency owners.</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>Consultant serving small agency owners specifically -- direct overlap with the agency-founder rows elsewhere in this sheet.</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>Hey Danielle — saw you're passionate about building systems for small businesses and helping agency owners specifically. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr"/>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Jill Hutchins</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Managing Consultant / Founder</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Your HR Partners -- boutique HR services</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jillhutchins/</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small, explicitly boutique HR consulting firm. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly 'boutique' self-positioning -- good qualitative size signal.</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jill — saw you run Your HR Partners as a boutique human resources services company. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr"/>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Scher</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Taylor Scher Consulting, LLC -- B2B SaaS SEO/content</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/taylorjosephscher/</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a B2B SaaS content/SEO consultancy who just hired employee #1 -- explicitly confirmed as a 2-person shop right now.</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly confirmed 2-person company (just crossed from solo to first hire) -- very high-confidence smallest-possible ICP fit.</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>Hey Taylor — saw you just onboarded your first full-time employee (an editorial manager) at Taylor Scher Consulting. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr"/>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Apoorv Sharma</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Found On AI -- AI search for B2B SaaS (Bengaluru)</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/apoorvshrm/</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small AI-search consultancy for B2B SaaS companies. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>AI-native small consultancy founder serving multiplayer's exact target client base.</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>Hey Apoorv — saw you're helping B2B SaaS companies with AI search visibility at Found On AI. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Anis Msakni</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Search &amp; AI Visibility Consultant</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- for B2B/SaaS companies</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>https://es.linkedin.com/in/anis-msakni-7b17991a9</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>Solo independent Search &amp; AI Visibility consultant for B2B/SaaS companies.</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>Solo consultant serving multiplayer's exact target client base -- purest form of the company-stage signal.</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>Hey Anis — saw you help B2B/SaaS companies grow visibility and revenue through SEO and AEO. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr"/>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Matt Craig</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Sheepdog Projects -- BI Consulting and Data Strategy</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mathieucraig/</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a small BI/data-strategy consultancy. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>Small consultancy founder in an underrepresented vertical (BI/analytics) for diversification.</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>Hey Matt — saw you co-founded Sheepdog Projects to offer BI consulting and data strategy services. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr"/>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Peter O'Donoghue</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Nynch -- growth platform for consultants and fractionals</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/peterodonoghue/</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small SaaS company building tools for the exact fractional-consultant audience heavily represented elsewhere in this sheet.</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>Small SaaS founder whose own customer base overlaps with many other rows in this sheet -- interesting potential channel as well as direct lead.</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>Hey Peter — saw you're building Nynch, a growth platform specifically for consultants and fractional professionals. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr"/>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Michael Twiddy</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Fame -- The B2B Podcast Agency</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/in/michael-twiddy-1a1391196</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small B2B podcast production agency, already discussing AI integration in the workflow.</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder already engaging with AI in production -- good adoption-readiness signal.</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>Hey Michael — saw you discuss AI integration in podcast production at Fame. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr"/>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Jason Bradwell</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>B2B Better -- podcast agency</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jason-bradwell-40b45751/</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small B2B podcast agency, publicly discussing AI in production. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder already engaging with AI in production -- good adoption-readiness signal.</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jason — saw you discuss how AI is being integrated into podcast production workflows at B2B Better. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr"/>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I109" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5801,6 +6761,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId128"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 13 more leads (140 total): video/creative, DevOps, fractional CMOs
Round 10: small video/animation studios serving SaaS and AI clients
(including one confirmed to have started as just two founders doing every
function), solo DevOps/AI-infrastructure consultants, and several fractional
CMOs/marketing consultancies -- the closest direct match to the marketing-ops
ICP in multiplayer-ai-context.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J129"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6646,9 +6646,585 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Dominic Noble</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Frogotiv -- animation/video studio</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/dominicnoble/</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small animation/video studio, explicitly confirmed to have started with just two founders doing every function themselves -- textbook wearing-every-hat ICP signal.</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed tiny founding team doing every function personally -- very high-confidence ICP fit on company stage and pain point.</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Hey Dominic — saw you and your co-founder originally handled strategy, storyboarding, illustration, animation, revisions, and client communication together at Frogotiv. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr"/>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Oyinkro K</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>K.OS VISUALS -- creative GTM partner for AI/SaaS companies</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/oyinkro-creativevideographer/</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small creative agency positioned specifically for AI/SaaS company clients.</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder serving multiplayer's exact target client base.</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>Hey Oyinkro — saw you're positioning K.OS VISUALS as a creative GTM partner for fast-growing AI/SaaS companies. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr"/>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Costin Modoianu</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Video Partner</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- video for SaaS &amp; Tech</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/costin-modoianu/</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Solo/small video production consultant specializing in SaaS and tech clients.</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>Solo consultant serving multiplayer's exact target client base.</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>Hey Costin — saw you turn complex SaaS products into clear, high-impact video as a strategic video partner. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr"/>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>Marek Bartík</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>pipetail.io -- AWS &amp; Kubernetes DevOps consulting</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/marekbartik/</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>Solo/small DevOps consultancy founder. Technical audience, likely an early adopter of new tooling.</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>Solo technical consultant -- purest form of the company-stage signal, strong early-adopter likelihood.</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>Hey Marek — saw you help companies adopt DevOps culture through on-site workshops and consulting at pipetail.io. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr"/>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>Michal Maxian</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Cloud Architecture consulting -- built a RAG platform for 15k+ users</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mmaxian/</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>AI &amp; Cloud Architect and founder of a small consultancy, hands-on building AI infrastructure himself.</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>Deeply technical AI-native founder -- strong thematic fit and early-adopter likelihood.</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>Hey Michal — saw you built a RAG platform for 15k+ users and now consult on DevOps culture and AI adoption. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr"/>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>Samuel Anderson-Levy</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CMO Agency (New York)</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/samuel-anderson-levy-33508528a/</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small fractional-CMO agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>Fractional marketing consultant -- direct fit with the marketing-ops ICP.</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>Hey Samuel — saw you run a fractional CMO agency in New York. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr"/>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>Joshua Kimber</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; Owner</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>sōsh -- fractional CMO / digital marketing agency</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/joshkimber/</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Founder/owner of a small fractional-CMO/digital-marketing agency. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>Small agency founder in the core marketing-ops ICP.</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Hey Joshua — saw you're driving data-driven growth for clients as founder of sōsh. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>Sara Pastor Ruprichova</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CMO</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>White Cloud Communications (Prague)</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/pastorsara/</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small strategic marketing consultancy serving growing businesses across Europe and beyond.</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>Fractional marketing consultant serving small businesses -- direct ICP fit.</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>Hey Sara — saw you help founders and SMEs turn marketing spend into measurable growth through White Cloud Communications. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr"/>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>Kristen Palmer</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder / CEO</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Boutique digital marketing consulting firm (B2B professional services)</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/kristenpalmer1/</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a small, self-described boutique marketing consultancy. Ex-Accenture.</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>Explicitly 'boutique' self-positioning -- good qualitative company-size signal.</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Hey Kristen — saw you co-founded a boutique full-service digital marketing consulting firm for B2B professional services. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr"/>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>Dawn Jacobs</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CMO</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- partners with early-stage founders/CEOs</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/dawnmjacobs/</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CMO explicitly partnering with early-stage founders. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>Fractional marketing consultant serving early-stage founders -- direct ICP fit.</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>Hey Dawn — saw you partner with early-stage founders and CEOs to build brands that scale. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr"/>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Jonny Butler</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CMO</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- strategy &amp; execution for early-stage B2B SaaS</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jonnybutler/</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CMO with direct in-house B2B SaaS marketing leadership experience, now serving early-stage SaaS clients.</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>Fractional marketing consultant with direct B2B SaaS operator background -- strong ICP and empathy fit.</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>Hey Jonny — saw you've been 3x Head of Marketing at B2B SaaS startups before going fractional. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>Hugo Pereira</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CGO/CMO</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Independent -- B2B SaaS &amp; deep tech</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/hugosbpereira/</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Fractional CGO/CMO for B2B SaaS and deep tech, author and previously exited founder himself.</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>Fractional consultant with founder-side empathy (previously exited a company himself) -- strong ICP fit.</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>Hey Hugo — saw you wrote "Teams in Hell" and are a 1x exited founder now doing fractional growth work. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr"/>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6781,6 +7357,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId140"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Reach 150 leads: final batch of YC W24 founders + AI-adoption consultants
Round 11 (final): 6 more YC W24 co-founders, plus AI-adoption consultants
whose own research/positioning closely mirrors multiplayer's thesis --
notably Marcus McGehee (The AI Consulting Lab), whose finding that only
~10% of a team actually uses AI tools 6 months after purchase is nearly
identical to the 'scattered, unused AI access' problem this product solves.

Sheet now totals 150 leads + 3 connectors, all sourced via
site:linkedin.com/in and site:linkedin.com/posts search this session --
no scraping, no login automation, consistent with the ToS constraints in
outreach-pipeline-context.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7222,9 +7222,489 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Annabell V.</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CTO</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>CoCrafter (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/annabell-v-86a73b227/</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CTO of a YC W24-batch startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage technical co-founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>Hey Annabell — saw you're co-founder and CTO of CoCrafter, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr"/>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>Nicole Atack</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Yarn (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nicole-atack-98194b2b8/</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W24-batch startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>Hey Nicole — saw you're co-founder of Yarn, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr"/>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>David Lalor</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>CEO &amp; Co-Founder</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Swift (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/davidlalor5/</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a YC W24-batch startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Hey David — saw you're CEO and co-founder of Swift, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr"/>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>Md Abdul Halim Rafi</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CTO</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Octolane AI (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/md-abdul-halim-rafi/</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CTO of a YC W24-batch AI startup -- confirmed very-early stage and directly AI-native.</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage AI founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>Hey Md — saw you're co-founder and CTO of Octolane AI, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr"/>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Joseph Palakapilly</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Meticulate (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jpalakapilly/</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W24-batch startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>Hey Joseph — saw you're co-founder of Meticulate, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr"/>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>Alex Choi</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Basalt Tech (Y Combinator W24)</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alex-choi/</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder of a YC W24-batch startup -- confirmed very-early stage.</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>YC-backed early-stage founder -- confirmed company stage.</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>Hey Alex — saw you co-founded Basalt Tech with Maximillian Bhatti, a YC W24 company. Quick question: across your team, does everyone end up using ChatGPT or Claude solo, with zero shared visibility into what anyone else tried or decided? That's the exact gap I'm building multiplayer for — a shared workspace where each person's AI agent posts its work into one thread the whole team can see and jump into. Rounding up a few small teams to test it free for 30-60 days in exchange for feedback — worth a quick look?</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr"/>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Marcus McGehee</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>The AI Consulting Lab</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/marcusmcgehee/</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small AI-adoption consultancy whose core finding -- that AI adoption fails on culture/training, not technology -- is nearly identical to multiplayer's own thesis about scattered, unused AI tool access.</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>Near-perfect thematic match: his own research names the exact 'AI tools bought but not actually adopted/shared' problem multiplayer is built to solve.</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Hey Marcus — saw your observation that companies buy AI licenses, announce it, and six months later only 10% of the team is actually using the tools. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr"/>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>Miranda Jones</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Founder / Lead Consultant</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>AI Consulting Network</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/miranda-jones-16a256115/</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small AI-adoption consultancy for small businesses. Headcount unconfirmed.</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>AI-adoption consultant serving multiplayer's exact target client base -- direct thematic fit.</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>Hey Miranda — saw you're empowering small businesses with AI tools and services through AI Consulting Network. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr"/>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>David MacKillop</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>MacKillop Solutions -- AI agent and automation consulting</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/david-mackillop/</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Founder of a small AI automation consultancy, hands-on building agent workflows for clients.</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>Technical AI-agent-building consultant -- strong thematic fit and early-adopter likelihood.</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>Hey David — saw you build intelligent workflows and AI agents using tools like n8n, Make.com, and Airtable. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr"/>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>Matthew Kuchera</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Mission AI Consulting</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/matthewkuchera/</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn only (no public email found)</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder/CEO of a small AI consultancy specifically focused on platform adoption and implementation -- exactly the failure mode multiplayer addresses.</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>AI-adoption specialist consultant -- near-direct thematic match with multiplayer's core value proposition.</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>Hey Matthew — saw you specialize in AI platform adoption and implementation at Mission AI Consulting. Curious if this resonates: across the small teams/clients you work with, is everyone using ChatGPT or Claude on their own, with no shared visibility into what got tried or decided? That's the gap I'm building multiplayer for — a shared workspace where a team's AI agents post their work into one thread instead of staying siloed in separate chats. Looking for a few small teams to test it free in exchange for feedback — think any of your clients (or you) would want an early look?</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr"/>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7369,6 +7849,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="rId150"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Strip self-referential framing from draft messages, pure questions only
Templates no longer say "I'm building" or "before building anything" or
reference multiplayer/a product at all. Each message is now just the
personal detail plus a direct question about how the person's team uses
AI and whether that usage is solo or shared.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -551,13 +551,13 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Hey Katheryn, saw you're running GROW Marketing Agency as a small, founder-led shop. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Katheryn, saw you're running GROW Marketing Agency as a small, founder-led shop. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -604,13 +604,13 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Hey Donna, saw your work bridging gaps and scaling teams as a startup RevOps operator. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Donna, saw your work bridging gaps and scaling teams as a startup RevOps operator. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -657,13 +657,13 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Hey Kristy, saw scaling GTM systems for B2B SaaS companies through your boutique RevOps consultancy. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Kristy, saw scaling GTM systems for B2B SaaS companies through your boutique RevOps consultancy. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -710,13 +710,13 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Hey Jackie, saw you run Digital Marketing Direction as a virtual HubSpot partner agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Jackie, saw you run Digital Marketing Direction as a virtual HubSpot partner agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -763,13 +763,13 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Hey Josephine, saw your Chief of Staff role spanning GTM, Operations, and AI. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Josephine, saw your Chief of Staff role spanning GTM, Operations, and AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -816,13 +816,13 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Hey Raj, saw you're running Goodman Lantern, a B2B content marketing agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Raj, saw you're running Goodman Lantern, a B2B content marketing agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -869,13 +869,13 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Hey Paul, saw you're co-founder and CPO of Spherecast, a YC S24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Paul, saw you're co-founder and CPO of Spherecast, a YC S24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -922,13 +922,13 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Hey Avi, saw you're co-founder of Shor, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Avi, saw you're co-founder of Shor, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -975,13 +975,13 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Hey Dhruv, saw you're co-founder of slashy.com, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Dhruv, saw you're co-founder of slashy.com, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1028,13 +1028,13 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Hey Michael, saw you're co-founder of AgentMail, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Michael, saw you're co-founder of AgentMail, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1081,13 +1081,13 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Hey Ishaan, saw you're co-founder of Omnara, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Ishaan, saw you're co-founder of Omnara, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1134,13 +1134,13 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Hey Raj, saw you're co-founder of Infinite, a YC W25 company, previously at Sardine. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Raj, saw you're co-founder of Infinite, a YC W25 company, previously at Sardine. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1187,13 +1187,13 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Hey Kushal, saw you're co-founder of Optifye.ai, a YC W25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Kushal, saw you're co-founder of Optifye.ai, a YC W25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1240,13 +1240,13 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Hey Nand, saw you're co-founder of Axal, a YC W25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Nand, saw you're co-founder of Axal, a YC W25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1293,13 +1293,13 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Hey William, saw you're co-founder of Janet AI, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey William, saw you're co-founder of Janet AI, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1346,13 +1346,13 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Hey Aditya, saw you're co-founder of Candor, a YC W25 company focused on insider-risk. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Aditya, saw you're co-founder of Candor, a YC W25 company focused on insider-risk. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1399,13 +1399,13 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Hey Chris, saw you're co-founder of Crustdata, a YC F24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Chris, saw you're co-founder of Crustdata, a YC F24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1452,13 +1452,13 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Hey Manmohit, saw you're co-founder of Crustdata, a YC F24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Manmohit, saw you're co-founder of Crustdata, a YC F24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1505,13 +1505,13 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Hey Shawn, saw you're co-founder and CEO of Penciled, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Shawn, saw you're co-founder and CEO of Penciled, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1558,13 +1558,13 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Hey Sarah, saw you're co-founder and COO of RetailReady, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Sarah, saw you're co-founder and COO of RetailReady, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1611,13 +1611,13 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Hey Chris, saw you're co-founder of Sonia, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Chris, saw you're co-founder of Sonia, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1664,13 +1664,13 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Hey William, saw you're co-founder of Centralize, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey William, saw you're co-founder of Centralize, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1717,13 +1717,13 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Hey Andy, saw you're co-founder and CEO of Respan, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Andy, saw you're co-founder and CEO of Respan, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1770,13 +1770,13 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Hey Givi, saw you're co-founder and CEO of KLIPY, a Techstars-backed company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Givi, saw you're co-founder and CEO of KLIPY, a Techstars-backed company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1823,13 +1823,13 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Hey Karla, saw you're co-founder and CEO of Shappi, a Techstars-backed company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Karla, saw you're co-founder and CEO of Shappi, a Techstars-backed company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1876,13 +1876,13 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Hey Moritz, saw you're co-founder of GEMESYS, a deeptech company with under 10 people. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Moritz, saw you're co-founder of GEMESYS, a deeptech company with under 10 people. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1929,13 +1929,13 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Hey Morrie, saw you're co-founder of Pingo, a YC S25 company with a team of just 3 people. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Morrie, saw you're co-founder of Pingo, a YC S25 company with a team of just 3 people. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -1982,13 +1982,13 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Hey Gurveer, saw you're co-founder and CEO of Certus AI, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Gurveer, saw you're co-founder and CEO of Certus AI, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2035,13 +2035,13 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Hey Alex, saw you're co-founder of Paloma, an AI-native CRM from YC S25. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Alex, saw you're co-founder of Paloma, an AI-native CRM from YC S25. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2088,13 +2088,13 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Hey Khalid, saw you've grown Munify to $20M ARR with a team of just 20 people. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Khalid, saw you've grown Munify to $20M ARR with a team of just 20 people. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2141,13 +2141,13 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Hey Arjun, saw you're co-founder of Knowlify, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Arjun, saw you're co-founder of Knowlify, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2194,13 +2194,13 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Hey Nazli, saw you're co-founder of Paloma, an AI-native CRM from YC S25. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Nazli, saw you're co-founder of Paloma, an AI-native CRM from YC S25. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2247,13 +2247,13 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Hey Neha, saw you're co-founder of Procindex, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Neha, saw you're co-founder of Procindex, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2300,13 +2300,13 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Hey John, saw you're co-founder of Autumn, a YC S25 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey John, saw you're co-founder of Autumn, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2353,13 +2353,13 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Hey Taylor, saw you just onboarded your first full-time employee (an editorial manager) at Taylor Scher Consulting. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Taylor, saw you just onboarded your first full-time employee (an editorial manager) at Taylor Scher Consulting. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2406,13 +2406,13 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Hey Dominic, saw you and your co-founder originally handled strategy, storyboarding, illustration, animation, revisions, and client communication together at Frogotiv. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Dominic, saw you and your co-founder originally handled strategy, storyboarding, illustration, animation, revisions, and client communication together at Frogotiv. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2459,13 +2459,13 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Hey Annabell, saw you're co-founder and CTO of CoCrafter, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Annabell, saw you're co-founder and CTO of CoCrafter, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2512,13 +2512,13 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Hey Nicole, saw you're co-founder of Yarn, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Nicole, saw you're co-founder of Yarn, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2565,13 +2565,13 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Hey David, saw you're CEO and co-founder of Swift, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey David, saw you're CEO and co-founder of Swift, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2618,13 +2618,13 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Hey Md, saw you're co-founder and CTO of Octolane AI, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Md, saw you're co-founder and CTO of Octolane AI, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2671,13 +2671,13 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Hey Joseph, saw you're co-founder of Meticulate, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Joseph, saw you're co-founder of Meticulate, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2724,13 +2724,13 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Hey Alex, saw you co-founded Basalt Tech with Maximillian Bhatti, a YC W24 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Alex, saw you co-founded Basalt Tech with Maximillian Bhatti, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2777,13 +2777,13 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Hey Elizabeth, saw you're running RevOps solo through PrecisionRevOps for multiple SaaS clients. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Elizabeth, saw you're running RevOps solo through PrecisionRevOps for multiple SaaS clients. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2830,13 +2830,13 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Hey Jeremy, saw you're juggling fractional RevOps/CRO roles across Rev, AgentSync, Ekho, and OperateWise at once. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Jeremy, saw you're juggling fractional RevOps/CRO roles across Rev, AgentSync, Ekho, and OperateWise at once. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2883,13 +2883,13 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Hey Haris, saw your recent post on what RevOps actually does and removing GTM silos. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Haris, saw your recent post on what RevOps actually does and removing GTM silos. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2936,13 +2936,13 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Hey Deepa, saw you're advising several high-growth startups at once as a fractional RevOps/strategy leader. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Deepa, saw you're advising several high-growth startups at once as a fractional RevOps/strategy leader. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2989,13 +2989,13 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Hey Mariya, saw you work as a fractional CFO across multiple early-stage B2B SaaS clients. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Mariya, saw you work as a fractional CFO across multiple early-stage B2B SaaS clients. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3042,13 +3042,13 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Hey John, saw the dozens of early-stage companies you've helped clean up CRM/HubSpot data at Sequoia Solutions. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey John, saw the dozens of early-stage companies you've helped clean up CRM/HubSpot data at Sequoia Solutions. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Hey Roberto, saw your posts on pipeline, forecasting, and AI at Revenue Hub Latam. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Roberto, saw your posts on pipeline, forecasting, and AI at Revenue Hub Latam. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3148,13 +3148,13 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Hey Johnathan, saw you built your own AI-powered social media tooling while running The SaaS Consultants. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Johnathan, saw you built your own AI-powered social media tooling while running The SaaS Consultants. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3201,13 +3201,13 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Hey Alex, saw you run your own solo HubSpot consulting practice. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Alex, saw you run your own solo HubSpot consulting practice. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3254,13 +3254,13 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Hey Ajay, saw you run MAWD Agency managing Google Ads, SEO, and websites for small businesses. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Ajay, saw you run MAWD Agency managing Google Ads, SEO, and websites for small businesses. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3307,13 +3307,13 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Hey Philip, saw you help companies use AI securely and purposefully as an independent consultant. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Philip, saw you help companies use AI securely and purposefully as an independent consultant. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3360,13 +3360,13 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Hey Oles, saw you're running Hey Digital, a performance marketing agency focused specifically on B2B SaaS. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Oles, saw you're running Hey Digital, a performance marketing agency focused specifically on B2B SaaS. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3413,13 +3413,13 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Hey Becky, saw you help small business owners get time back through BK's Bookkeeping. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Becky, saw you help small business owners get time back through BK's Bookkeeping. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3466,13 +3466,13 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Hey Tom, saw you're part of an AI Mastermind group applying tech-forward solutions to bookkeeping. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Tom, saw you're part of an AI Mastermind group applying tech-forward solutions to bookkeeping. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3519,13 +3519,13 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Hey Michael, saw you're running Boldly with a small team of creative minds. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Michael, saw you're running Boldly with a small team of creative minds. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3572,13 +3572,13 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Hey Michael, saw you're co-founder and de-facto Operations Manager at 10X ERP. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Michael, saw you're co-founder and de-facto Operations Manager at 10X ERP. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3625,13 +3625,13 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Hey Pavels, saw you're targeting B2B SaaS founders specifically through Camel Digital. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Pavels, saw you're targeting B2B SaaS founders specifically through Camel Digital. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3678,13 +3678,13 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Hey Aaron, saw your work helping brands scale with strategic video content and AI repurposing. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Aaron, saw your work helping brands scale with strategic video content and AI repurposing. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3731,13 +3731,13 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Hey Ebru, saw your take that AI translating doesn't mean localization is solved. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Ebru, saw your take that AI translating doesn't mean localization is solved. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3784,13 +3784,13 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Hey Crystal, saw you help SaaS founders and CS teams with customer success operations as a fractional consultant. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Crystal, saw you help SaaS founders and CS teams with customer success operations as a fractional consultant. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3837,13 +3837,13 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Hey Jamiu, saw you're running Hidden Gems, focused on creator-led growth specifically for B2B AI &amp; SaaS companies. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Jamiu, saw you're running Hidden Gems, focused on creator-led growth specifically for B2B AI &amp; SaaS companies. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3890,13 +3890,13 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Hey Harry, saw you're building 'mate,' an AI growth teammate for small businesses. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Harry, saw you're building 'mate,' an AI growth teammate for small businesses. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3943,13 +3943,13 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Hey Mihai, saw you're building MspCoreX to replace fragmented MSP tool stacks with one intelligent core. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Mihai, saw you're building MspCoreX to replace fragmented MSP tool stacks with one intelligent core. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3996,13 +3996,13 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Hey Michelle, saw your mission of helping small and mid-sized agencies grow through Real Marketing Muscle. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Michelle, saw your mission of helping small and mid-sized agencies grow through Real Marketing Muscle. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4049,13 +4049,13 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>Hey Austin, saw you're making AI accessible and practical for entrepreneurs and small business owners at digital3 AI. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Austin, saw you're making AI accessible and practical for entrepreneurs and small business owners at digital3 AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4102,13 +4102,13 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>Hey Yael, saw you built an AI agent trained on multiple brand voices and content formats at Ashley Digital. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Yael, saw you built an AI agent trained on multiple brand voices and content formats at Ashley Digital. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4155,13 +4155,13 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>Hey Ai, saw you're democratizing access to AI and no-code tools for individuals and small businesses through Common AI. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Ai, saw you're democratizing access to AI and no-code tools for individuals and small businesses through Common AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4208,13 +4208,13 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Hey Vanhishikha, saw you've partnered with 100+ B2B SaaS companies on SEO and content through Contensify. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Vanhishikha, saw you've partnered with 100+ B2B SaaS companies on SEO and content through Contensify. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr"/>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4261,13 +4261,13 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>Hey Susan, saw you help founders build self-sufficient teams as a People Ops &amp; Systems consultant. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Susan, saw you help founders build self-sufficient teams as a People Ops &amp; Systems consultant. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4314,13 +4314,13 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>Hey Heidi, saw you focus on People Ops/HR solutions specifically for startups and tech companies. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Heidi, saw you focus on People Ops/HR solutions specifically for startups and tech companies. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr"/>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4367,13 +4367,13 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>Hey Michelle, saw you provide scalable HR systems for growing teams through Quantum People Ops. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Michelle, saw you provide scalable HR systems for growing teams through Quantum People Ops. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4420,13 +4420,13 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>Hey Danielle, saw you're passionate about building systems for small businesses and helping agency owners specifically. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Danielle, saw you're passionate about building systems for small businesses and helping agency owners specifically. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4473,13 +4473,13 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>Hey Anis, saw you help B2B/SaaS companies grow visibility and revenue through SEO and AEO. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Anis, saw you help B2B/SaaS companies grow visibility and revenue through SEO and AEO. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4526,13 +4526,13 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>Hey Peter, saw you're building Nynch, a growth platform specifically for consultants and fractional professionals. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Peter, saw you're building Nynch, a growth platform specifically for consultants and fractional professionals. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4579,13 +4579,13 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>Hey Michael, saw you discuss AI integration in podcast production at Fame. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Michael, saw you discuss AI integration in podcast production at Fame. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4632,13 +4632,13 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>Hey Oyinkro, saw you're positioning K.OS VISUALS as a creative GTM partner for fast-growing AI/SaaS companies. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Oyinkro, saw you're positioning K.OS VISUALS as a creative GTM partner for fast-growing AI/SaaS companies. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4685,13 +4685,13 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Hey Costin, saw you turn complex SaaS products into clear, high-impact video as a strategic video partner. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Costin, saw you turn complex SaaS products into clear, high-impact video as a strategic video partner. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4738,13 +4738,13 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>Hey Marek, saw you help companies adopt DevOps culture through on-site workshops and consulting at pipetail.io. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Marek, saw you help companies adopt DevOps culture through on-site workshops and consulting at pipetail.io. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4791,13 +4791,13 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Hey Michal, saw you built a RAG platform for 15k+ users and now consult on DevOps culture and AI adoption. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Michal, saw you built a RAG platform for 15k+ users and now consult on DevOps culture and AI adoption. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4844,13 +4844,13 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Hey Sara, saw you help founders and SMEs turn marketing spend into measurable growth through White Cloud Communications. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Sara, saw you help founders and SMEs turn marketing spend into measurable growth through White Cloud Communications. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr"/>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4897,13 +4897,13 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>Hey Jonny, saw you've been 3x Head of Marketing at B2B SaaS startups before going fractional. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Jonny, saw you've been 3x Head of Marketing at B2B SaaS startups before going fractional. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -4950,13 +4950,13 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>Hey Hugo, saw you wrote "Teams in Hell" and are a 1x exited founder now doing fractional growth work. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Hugo, saw you wrote "Teams in Hell" and are a 1x exited founder now doing fractional growth work. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5003,13 +5003,13 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>Hey Marcus, saw your observation that companies buy AI licenses, announce it, and six months later only 10% of the team is actually using the tools. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Marcus, saw your observation that companies buy AI licenses, announce it, and six months later only 10% of the team is actually using the tools. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5056,13 +5056,13 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>Hey David, saw you build intelligent workflows and AI agents using tools like n8n, Make.com, and Airtable. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey David, saw you build intelligent workflows and AI agents using tools like n8n, Make.com, and Airtable. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr"/>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5109,13 +5109,13 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>Hey Matthew, saw you specialize in AI platform adoption and implementation at Mission AI Consulting. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Matthew, saw you specialize in AI platform adoption and implementation at Mission AI Consulting. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5162,13 +5162,13 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>Hey Adam, saw you've built a lean senior team at Growth Union for early-stage B2B SaaS clients like Writer and Recorded Future. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Adam, saw you've built a lean senior team at Growth Union for early-stage B2B SaaS clients like Writer and Recorded Future. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr"/>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5215,13 +5215,13 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>Hey David, saw you're building Lynx Growth Agency around AI-driven marketing and automation. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey David, saw you're building Lynx Growth Agency around AI-driven marketing and automation. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5268,13 +5268,13 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>Hey Alex, saw your writing on AI agents in RevOps as CEO of Forecastio. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Alex, saw your writing on AI agents in RevOps as CEO of Forecastio. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr"/>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5321,13 +5321,13 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Hey Kristofer, saw your tagline about helping startups supercharge their small RevOps teams. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Kristofer, saw your tagline about helping startups supercharge their small RevOps teams. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr"/>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5374,13 +5374,13 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>Hey Shaun, saw you're building agentic AI systems as an AI Marketing Engineer while running thisisagency.ai. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Shaun, saw you're building agentic AI systems as an AI Marketing Engineer while running thisisagency.ai. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J93" s="2" t="inlineStr"/>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5427,13 +5427,13 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>Hey Sam, saw you're running Origin 63 as a small, results-focused growth agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Sam, saw you're running Origin 63 as a small, results-focused growth agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr"/>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5480,13 +5480,13 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>Hey Josh, saw your work on revenue growth and retention at Hüify, a HubSpot partner agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Josh, saw your work on revenue growth and retention at Hüify, a HubSpot partner agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr"/>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5533,13 +5533,13 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>Hey Clwyd, saw you work as an AI consultant at Whitehat, helping businesses adopt AI. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Clwyd, saw you work as an AI consultant at Whitehat, helping businesses adopt AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr"/>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5586,13 +5586,13 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>Hey Clara, saw you're employee #3 and Chief of Staff at Kairos. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Clara, saw you're employee #3 and Chief of Staff at Kairos. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr"/>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5639,13 +5639,13 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>Hey Riddhi, saw you're running Thought In A Dot as a content marketing agency and brand strategist. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Riddhi, saw you're running Thought In A Dot as a content marketing agency and brand strategist. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr"/>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5692,13 +5692,13 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>Hey John, saw you founded Creative Engine, a branding and digital marketing agency in Austin. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey John, saw you founded Creative Engine, a branding and digital marketing agency in Austin. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr"/>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5745,13 +5745,13 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>Hey Laney, saw you run The Design Boutique and pride yourselves on being able to pivot quickly as a small shop. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Laney, saw you run The Design Boutique and pride yourselves on being able to pivot quickly as a small shop. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr"/>
       <c r="K100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5798,13 +5798,13 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>Hey Thomas, saw you founded Venture Visuals, a creative agency in Seattle. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Thomas, saw you founded Venture Visuals, a creative agency in Seattle. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr"/>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5851,13 +5851,13 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>Hey Santosh, saw you're running Visual Best, an AI creative production agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Santosh, saw you're running Visual Best, an AI creative production agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr"/>
       <c r="K102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5904,13 +5904,13 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>Hey David, saw you describe your business as having an AI-first mindset while running Sounds Good Agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey David, saw you describe your business as having an AI-first mindset while running Sounds Good Agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr"/>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -5957,13 +5957,13 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>Hey Mark, saw you're a pioneer in AI-native software engineering as founder of SoftwareFactory.ai. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Mark, saw you're a pioneer in AI-native software engineering as founder of SoftwareFactory.ai. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr"/>
       <c r="K104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6010,13 +6010,13 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>Hey Dylan, saw you install AI systems into service businesses as an independent consultant. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Dylan, saw you install AI systems into service businesses as an independent consultant. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr"/>
       <c r="K105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6063,13 +6063,13 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>Hey Alex, saw you're co-founder/CEO of Intryc, a Y Combinator S24 startup. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Alex, saw you're co-founder/CEO of Intryc, a Y Combinator S24 startup. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr"/>
       <c r="K106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6116,13 +6116,13 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>Hey Arham, saw you founded Pixated, a performance marketing agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Arham, saw you founded Pixated, a performance marketing agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr"/>
       <c r="K107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6169,13 +6169,13 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>Hey Alex, saw you're scaling DTC ecommerce brands through Tierra. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Alex, saw you're scaling DTC ecommerce brands through Tierra. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr"/>
       <c r="K108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6222,13 +6222,13 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>Hey Beckie, saw you run a boutique recruiting agency with a niche sector focus. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Beckie, saw you run a boutique recruiting agency with a niche sector focus. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr"/>
       <c r="K109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6275,13 +6275,13 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>Hey Katie, saw your writing on balancing technology and human connection in recruiting at CollabRecruit. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Katie, saw your writing on balancing technology and human connection in recruiting at CollabRecruit. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr"/>
       <c r="K110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6328,13 +6328,13 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>Hey Jennifer, saw you founded Bookkeeping Done Right to serve small and medium businesses in South Florida. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Jennifer, saw you founded Bookkeeping Done Right to serve small and medium businesses in South Florida. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr"/>
       <c r="K111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6381,13 +6381,13 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>Hey Parry, saw you're leading a team of senior PR leaders at Crackle PR. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Parry, saw you're leading a team of senior PR leaders at Crackle PR. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr"/>
       <c r="K112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6434,13 +6434,13 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>Hey Carin, saw your writing on AI strategy in communications. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Carin, saw your writing on AI strategy in communications. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr"/>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6487,13 +6487,13 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>Hey Erika, saw you're running 85th &amp; Park, a culture-driven creative marketing and comms agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Erika, saw you're running 85th &amp; Park, a culture-driven creative marketing and comms agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr"/>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6540,13 +6540,13 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>Hey Sam, saw you just founded a new AI automation agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Sam, saw you just founded a new AI automation agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr"/>
       <c r="K115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6593,13 +6593,13 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>Hey M, saw you're running your own web design agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey M, saw you're running your own web design agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr"/>
       <c r="K116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6646,13 +6646,13 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>Hey Kristen, saw your interest in AI adoption for web design and development. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Kristen, saw your interest in AI adoption for web design and development. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr"/>
       <c r="K117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6699,13 +6699,13 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>Hey Stefen, saw you co-founded Kelp Creative Agency. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Stefen, saw you co-founded Kelp Creative Agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr"/>
       <c r="K118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6752,13 +6752,13 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>Hey Dean, saw you're co-founder and Head of Operations at Superstate. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Dean, saw you're co-founder and Head of Operations at Superstate. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr"/>
       <c r="K119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6805,13 +6805,13 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>Hey Leah, saw you're co-founder and Head of Operations at See Jane Drill. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Leah, saw you're co-founder and Head of Operations at See Jane Drill. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr"/>
       <c r="K120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6858,13 +6858,13 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>Hey Evan, saw you're using AI tools like Heygen and Freepik at Boomin' Brands Media. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Evan, saw you're using AI tools like Heygen and Freepik at Boomin' Brands Media. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr"/>
       <c r="K121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6911,13 +6911,13 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>Hey Yash, saw your AI-led creative production work at Lemonade Creatives. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Yash, saw your AI-led creative production work at Lemonade Creatives. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr"/>
       <c r="K122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6964,13 +6964,13 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
-          <t>Hey Adam, saw you built Taia, a workflow system addressing friction in translation processes. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Adam, saw you built Taia, a workflow system addressing friction in translation processes. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J123" s="2" t="inlineStr"/>
       <c r="K123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7017,13 +7017,13 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>Hey Adriana, saw you run Libre Design Studio specifically for founders and startups. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Adriana, saw you run Libre Design Studio specifically for founders and startups. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr"/>
       <c r="K124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7070,13 +7070,13 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>Hey Atiqur, saw you founded Design Monks. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Atiqur, saw you founded Design Monks. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr"/>
       <c r="K125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7123,13 +7123,13 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>Hey Thomas, saw you help B2B SaaS companies turn Customer Success into measurable revenue at Revora Consultants. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Thomas, saw you help B2B SaaS companies turn Customer Success into measurable revenue at Revora Consultants. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr"/>
       <c r="K126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7176,13 +7176,13 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>Hey Peter, saw you're building Trendin, an AI-native operating system for influencer agencies. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Peter, saw you're building Trendin, an AI-native operating system for influencer agencies. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr"/>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7229,13 +7229,13 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>Hey Krishna, saw you built LegalConnect to deliver AI-drafted, solicitor-reviewed legal documents for SMEs. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Krishna, saw you built LegalConnect to deliver AI-drafted, solicitor-reviewed legal documents for SMEs. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr"/>
       <c r="K128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7282,13 +7282,13 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>Hey Jay, saw you run Startup Legal Group, serving startup clients directly. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Jay, saw you run Startup Legal Group, serving startup clients directly. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J129" s="2" t="inlineStr"/>
       <c r="K129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7335,13 +7335,13 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>Hey Nahme, saw you're running Research Connections, a market research consulting and field management company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Nahme, saw you're running Research Connections, a market research consulting and field management company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr"/>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7388,13 +7388,13 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>Hey Jake, saw you run JakeWu Market Research, a small solo-founder shop. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Jake, saw you run JakeWu Market Research, a small solo-founder shop. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr"/>
       <c r="K131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7441,13 +7441,13 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>Hey Jenna, saw you founded an education platform teaching interior designers to use AI. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Jenna, saw you founded an education platform teaching interior designers to use AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr"/>
       <c r="K132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7494,13 +7494,13 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>Hey Nina, saw you co-founded Curioso, an assemblage of designers, architects, and business-minded creatives. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Nina, saw you co-founded Curioso, an assemblage of designers, architects, and business-minded creatives. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J133" s="2" t="inlineStr"/>
       <c r="K133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7547,13 +7547,13 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>Hey Snehadeep, saw you use AI-driven design tools as founder of Studio ORCHIVIZ. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Snehadeep, saw you use AI-driven design tools as founder of Studio ORCHIVIZ. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr"/>
       <c r="K134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7600,13 +7600,13 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>Hey Akeem, saw you're co-founder of Thread, a YC W23 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Akeem, saw you're co-founder of Thread, a YC W23 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J135" s="2" t="inlineStr"/>
       <c r="K135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7653,13 +7653,13 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>Hey Ty, saw you're co-founder and CEO of inBuild, a YC W23 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Ty, saw you're co-founder and CEO of inBuild, a YC W23 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr"/>
       <c r="K136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7706,13 +7706,13 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>Hey Vlad, saw you're co-founder of Infisical, a YC W23 company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Vlad, saw you're co-founder of Infisical, a YC W23 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr"/>
       <c r="K137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7759,13 +7759,13 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>Hey Neel, saw you're co-founder of Clueso, an AI video creation company from YC W23. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Neel, saw you're co-founder of Clueso, an AI video creation company from YC W23. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr"/>
       <c r="K138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7812,13 +7812,13 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>Hey Sourav, saw you focus on brand strategy specifically for early-stage startups at Branded Minds. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Sourav, saw you focus on brand strategy specifically for early-stage startups at Branded Minds. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr"/>
       <c r="K139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7865,13 +7865,13 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>Hey Ulli, saw you run First The Trousers as a brand strategy and positioning consultancy. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Ulli, saw you run First The Trousers as a brand strategy and positioning consultancy. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr"/>
       <c r="K140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7918,13 +7918,13 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>Hey Lance, saw you're building BrandChef.ai. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Lance, saw you're building BrandChef.ai. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr"/>
       <c r="K141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -7971,13 +7971,13 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>Hey Branden, saw you founded Build, a branding agency built around practical design. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Branden, saw you founded Build, a branding agency built around practical design. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr"/>
       <c r="K142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8024,13 +8024,13 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>Hey Jill, saw you run Your HR Partners as a boutique human resources services company. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Jill, saw you run Your HR Partners as a boutique human resources services company. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr"/>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8077,13 +8077,13 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>Hey Apoorv, saw you're helping B2B SaaS companies with AI search visibility at Found On AI. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Apoorv, saw you're helping B2B SaaS companies with AI search visibility at Found On AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr"/>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8130,13 +8130,13 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>Hey Matt, saw you co-founded Sheepdog Projects to offer BI consulting and data strategy services. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Matt, saw you co-founded Sheepdog Projects to offer BI consulting and data strategy services. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr"/>
       <c r="K145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8183,13 +8183,13 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>Hey Jason, saw you discuss how AI is being integrated into podcast production workflows at B2B Better. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Jason, saw you discuss how AI is being integrated into podcast production workflows at B2B Better. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr"/>
       <c r="K146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8236,13 +8236,13 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>Hey Samuel, saw you run a fractional CMO agency in New York. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Samuel, saw you run a fractional CMO agency in New York. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr"/>
       <c r="K147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8289,13 +8289,13 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>Hey Joshua, saw you're driving data-driven growth for clients as founder of sōsh. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Joshua, saw you're driving data-driven growth for clients as founder of sōsh. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr"/>
       <c r="K148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8342,13 +8342,13 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>Hey Kristen, saw you co-founded a boutique full-service digital marketing consulting firm for B2B professional services. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across your team, does everyone end up using ChatGPT or Claude on their own, or is there any shared visibility into what people are trying or deciding? Would you be open to a quick chat about how your team handles it?</t>
+          <t>Hey Kristen, saw you co-founded a boutique full-service digital marketing consulting firm for B2B professional services. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr"/>
       <c r="K149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8395,13 +8395,13 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>Hey Dawn, saw you partner with early-stage founders and CEOs to build brands that scale. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Dawn, saw you partner with early-stage founders and CEOs to build brands that scale. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr"/>
       <c r="K150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8448,13 +8448,13 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>Hey Miranda, saw you're empowering small businesses with AI tools and services through AI Consulting Network. I'm looking into how small teams actually use AI day to day before building anything. Quick question: across the teams or clients you work with, is AI tool usage mostly solo, or is there any shared visibility into what's being tried? Would love your read, open to a quick chat?</t>
+          <t>Hey Miranda, saw you're empowering small businesses with AI tools and services through AI Consulting Network. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr"/>
       <c r="K151" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8742,13 +8742,13 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Hey Darrell, saw your newsletter on marketing ops team structure and career growth. I'm researching how small ops teams actually use AI day to day, not pitching anything yet. Curious whether solo AI usage with little shared visibility across a team is a theme you hear from your community. Open to a quick chat, and happy to share back whatever I learn.</t>
+          <t>Hey Darrell, saw your newsletter on marketing ops team structure and career growth. Question for you: is solo AI tool usage with little shared visibility across a team something you hear about often from your community? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8795,13 +8795,13 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Hey Jen, saw your weekly newsletter for the marketing ops community. I'm researching how small ops teams actually use AI day to day, not pitching anything yet. Curious whether solo AI usage with little shared visibility across a team is a theme you hear from your community. Open to a quick chat, and happy to share back whatever I learn.</t>
+          <t>Hey Jen, saw your weekly newsletter for the marketing ops community. Question for you: is solo AI tool usage with little shared visibility across a team something you hear about often from your community? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -8848,13 +8848,13 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Hey Mike, saw MO Pros hitting 4,000+ marketing/RevOps members. I'm researching how small ops teams actually use AI day to day, not pitching anything yet. Curious whether solo AI usage with little shared visibility across a team is a theme you hear from your community. Open to a quick chat, and happy to share back whatever I learn.</t>
+          <t>Hey Mike, saw MO Pros hitting 4,000+ marketing/RevOps members. Question for you: is solo AI tool usage with little shared visibility across a team something you hear about often from your community? Curious what you're seeing.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a Subject line for each message
New Subject column (kind-based: team/AI, clients/AI, or community/AI),
same no-product framing as the message body. Only matters for LinkedIn
InMail (messaging outside your network); safe to ignore on a message to
an existing 1st-degree connection, which has no subject field.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwV72oFmQcGr6gPLgH4BT8
</commit_message>
<xml_diff>
--- a/outreach/leads.xlsx
+++ b/outreach/leads.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K151"/>
+  <dimension ref="A1:L151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -446,9 +446,10 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="65" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,15 +495,20 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Draft Message</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Date Found</t>
         </is>
@@ -551,11 +557,16 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Hey Katheryn, saw you're running GROW Marketing Agency as a small, founder-led shop. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -604,11 +615,16 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>Hey Donna, saw your work bridging gaps and scaling teams as a startup RevOps operator. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -657,11 +673,16 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>Hey Kristy, saw scaling GTM systems for B2B SaaS companies through your boutique RevOps consultancy. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -710,11 +731,16 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
           <t>Hey Jackie, saw you run Digital Marketing Direction as a virtual HubSpot partner agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -763,11 +789,16 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>Hey Josephine, saw your Chief of Staff role spanning GTM, Operations, and AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -816,11 +847,16 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
           <t>Hey Raj, saw you're running Goodman Lantern, a B2B content marketing agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -869,11 +905,16 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>Hey Paul, saw you're co-founder and CPO of Spherecast, a YC S24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -922,11 +963,16 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
           <t>Hey Avi, saw you're co-founder of Shor, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -975,11 +1021,16 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
           <t>Hey Dhruv, saw you're co-founder of slashy.com, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1028,11 +1079,16 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
           <t>Hey Michael, saw you're co-founder of AgentMail, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1081,11 +1137,16 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
           <t>Hey Ishaan, saw you're co-founder of Omnara, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1134,11 +1195,16 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
           <t>Hey Raj, saw you're co-founder of Infinite, a YC W25 company, previously at Sardine. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1187,11 +1253,16 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
           <t>Hey Kushal, saw you're co-founder of Optifye.ai, a YC W25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1240,11 +1311,16 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
           <t>Hey Nand, saw you're co-founder of Axal, a YC W25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1293,11 +1369,16 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
           <t>Hey William, saw you're co-founder of Janet AI, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1346,11 +1427,16 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
           <t>Hey Aditya, saw you're co-founder of Candor, a YC W25 company focused on insider-risk. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1399,11 +1485,16 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
           <t>Hey Chris, saw you're co-founder of Crustdata, a YC F24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1452,11 +1543,16 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
           <t>Hey Manmohit, saw you're co-founder of Crustdata, a YC F24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1505,11 +1601,16 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
           <t>Hey Shawn, saw you're co-founder and CEO of Penciled, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1558,11 +1659,16 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
           <t>Hey Sarah, saw you're co-founder and COO of RetailReady, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1611,11 +1717,16 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
           <t>Hey Chris, saw you're co-founder of Sonia, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1664,11 +1775,16 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
           <t>Hey William, saw you're co-founder of Centralize, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1717,11 +1833,16 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
           <t>Hey Andy, saw you're co-founder and CEO of Respan, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1770,11 +1891,16 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
           <t>Hey Givi, saw you're co-founder and CEO of KLIPY, a Techstars-backed company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1823,11 +1949,16 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
           <t>Hey Karla, saw you're co-founder and CEO of Shappi, a Techstars-backed company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1876,11 +2007,16 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
           <t>Hey Moritz, saw you're co-founder of GEMESYS, a deeptech company with under 10 people. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1929,11 +2065,16 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
           <t>Hey Morrie, saw you're co-founder of Pingo, a YC S25 company with a team of just 3 people. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -1982,11 +2123,16 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
           <t>Hey Gurveer, saw you're co-founder and CEO of Certus AI, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2035,11 +2181,16 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
           <t>Hey Alex, saw you're co-founder of Paloma, an AI-native CRM from YC S25. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2088,11 +2239,16 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
           <t>Hey Khalid, saw you've grown Munify to $20M ARR with a team of just 20 people. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2141,11 +2297,16 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
           <t>Hey Arjun, saw you're co-founder of Knowlify, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2194,11 +2355,16 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
           <t>Hey Nazli, saw you're co-founder of Paloma, an AI-native CRM from YC S25. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2247,11 +2413,16 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
           <t>Hey Neha, saw you're co-founder of Procindex, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2300,11 +2471,16 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
           <t>Hey John, saw you're co-founder of Autumn, a YC S25 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2353,11 +2529,16 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
           <t>Hey Taylor, saw you just onboarded your first full-time employee (an editorial manager) at Taylor Scher Consulting. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2406,11 +2587,16 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
           <t>Hey Dominic, saw you and your co-founder originally handled strategy, storyboarding, illustration, animation, revisions, and client communication together at Frogotiv. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2459,11 +2645,16 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
           <t>Hey Annabell, saw you're co-founder and CTO of CoCrafter, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2512,11 +2703,16 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
           <t>Hey Nicole, saw you're co-founder of Yarn, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2565,11 +2761,16 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
           <t>Hey David, saw you're CEO and co-founder of Swift, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2618,11 +2819,16 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
           <t>Hey Md, saw you're co-founder and CTO of Octolane AI, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2671,11 +2877,16 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
           <t>Hey Joseph, saw you're co-founder of Meticulate, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2724,11 +2935,16 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
           <t>Hey Alex, saw you co-founded Basalt Tech with Maximillian Bhatti, a YC W24 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2777,11 +2993,16 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
           <t>Hey Elizabeth, saw you're running RevOps solo through PrecisionRevOps for multiple SaaS clients. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr"/>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2830,11 +3051,16 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
           <t>Hey Jeremy, saw you're juggling fractional RevOps/CRO roles across Rev, AgentSync, Ekho, and OperateWise at once. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2883,11 +3109,16 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
           <t>Hey Haris, saw your recent post on what RevOps actually does and removing GTM silos. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2936,11 +3167,16 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
           <t>Hey Deepa, saw you're advising several high-growth startups at once as a fractional RevOps/strategy leader. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr"/>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -2989,11 +3225,16 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
           <t>Hey Mariya, saw you work as a fractional CFO across multiple early-stage B2B SaaS clients. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr"/>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3042,11 +3283,16 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
           <t>Hey John, saw the dozens of early-stage companies you've helped clean up CRM/HubSpot data at Sequoia Solutions. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr"/>
-      <c r="K49" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3095,11 +3341,16 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
           <t>Hey Roberto, saw your posts on pipeline, forecasting, and AI at Revenue Hub Latam. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr"/>
-      <c r="K50" s="2" t="inlineStr">
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3148,11 +3399,16 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
           <t>Hey Johnathan, saw you built your own AI-powered social media tooling while running The SaaS Consultants. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr"/>
-      <c r="K51" s="2" t="inlineStr">
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3201,11 +3457,16 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
           <t>Hey Alex, saw you run your own solo HubSpot consulting practice. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr"/>
-      <c r="K52" s="2" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3254,11 +3515,16 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
           <t>Hey Ajay, saw you run MAWD Agency managing Google Ads, SEO, and websites for small businesses. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr"/>
-      <c r="K53" s="2" t="inlineStr">
+      <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3307,11 +3573,16 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
           <t>Hey Philip, saw you help companies use AI securely and purposefully as an independent consultant. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr"/>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3360,11 +3631,16 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
           <t>Hey Oles, saw you're running Hey Digital, a performance marketing agency focused specifically on B2B SaaS. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr"/>
-      <c r="K55" s="2" t="inlineStr">
+      <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3413,11 +3689,16 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
           <t>Hey Becky, saw you help small business owners get time back through BK's Bookkeeping. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr"/>
-      <c r="K56" s="2" t="inlineStr">
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3466,11 +3747,16 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
           <t>Hey Tom, saw you're part of an AI Mastermind group applying tech-forward solutions to bookkeeping. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr"/>
-      <c r="K57" s="2" t="inlineStr">
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3519,11 +3805,16 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
           <t>Hey Michael, saw you're running Boldly with a small team of creative minds. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J58" s="2" t="inlineStr"/>
-      <c r="K58" s="2" t="inlineStr">
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3572,11 +3863,16 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
           <t>Hey Michael, saw you're co-founder and de-facto Operations Manager at 10X ERP. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr"/>
-      <c r="K59" s="2" t="inlineStr">
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3625,11 +3921,16 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
           <t>Hey Pavels, saw you're targeting B2B SaaS founders specifically through Camel Digital. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr">
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3678,11 +3979,16 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
           <t>Hey Aaron, saw your work helping brands scale with strategic video content and AI repurposing. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr">
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3731,11 +4037,16 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
           <t>Hey Ebru, saw your take that AI translating doesn't mean localization is solved. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr">
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3784,11 +4095,16 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
           <t>Hey Crystal, saw you help SaaS founders and CS teams with customer success operations as a fractional consultant. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr"/>
-      <c r="K63" s="2" t="inlineStr">
+      <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3837,11 +4153,16 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
           <t>Hey Jamiu, saw you're running Hidden Gems, focused on creator-led growth specifically for B2B AI &amp; SaaS companies. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr"/>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3890,11 +4211,16 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
           <t>Hey Harry, saw you're building 'mate,' an AI growth teammate for small businesses. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr"/>
-      <c r="K65" s="2" t="inlineStr">
+      <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3943,11 +4269,16 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
           <t>Hey Mihai, saw you're building MspCoreX to replace fragmented MSP tool stacks with one intelligent core. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr"/>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -3996,11 +4327,16 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
           <t>Hey Michelle, saw your mission of helping small and mid-sized agencies grow through Real Marketing Muscle. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr"/>
-      <c r="K67" s="2" t="inlineStr">
+      <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4049,11 +4385,16 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
           <t>Hey Austin, saw you're making AI accessible and practical for entrepreneurs and small business owners at digital3 AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr"/>
-      <c r="K68" s="2" t="inlineStr">
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4102,11 +4443,16 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
           <t>Hey Yael, saw you built an AI agent trained on multiple brand voices and content formats at Ashley Digital. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr"/>
-      <c r="K69" s="2" t="inlineStr">
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4155,11 +4501,16 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
           <t>Hey Ai, saw you're democratizing access to AI and no-code tools for individuals and small businesses through Common AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr"/>
-      <c r="K70" s="2" t="inlineStr">
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4208,11 +4559,16 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
           <t>Hey Vanhishikha, saw you've partnered with 100+ B2B SaaS companies on SEO and content through Contensify. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J71" s="2" t="inlineStr"/>
-      <c r="K71" s="2" t="inlineStr">
+      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4261,11 +4617,16 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
           <t>Hey Susan, saw you help founders build self-sufficient teams as a People Ops &amp; Systems consultant. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J72" s="2" t="inlineStr"/>
-      <c r="K72" s="2" t="inlineStr">
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4314,11 +4675,16 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
           <t>Hey Heidi, saw you focus on People Ops/HR solutions specifically for startups and tech companies. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J73" s="2" t="inlineStr"/>
-      <c r="K73" s="2" t="inlineStr">
+      <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4367,11 +4733,16 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
           <t>Hey Michelle, saw you provide scalable HR systems for growing teams through Quantum People Ops. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J74" s="2" t="inlineStr"/>
-      <c r="K74" s="2" t="inlineStr">
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4420,11 +4791,16 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
           <t>Hey Danielle, saw you're passionate about building systems for small businesses and helping agency owners specifically. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J75" s="2" t="inlineStr"/>
-      <c r="K75" s="2" t="inlineStr">
+      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4473,11 +4849,16 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
           <t>Hey Anis, saw you help B2B/SaaS companies grow visibility and revenue through SEO and AEO. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr"/>
-      <c r="K76" s="2" t="inlineStr">
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4526,11 +4907,16 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
           <t>Hey Peter, saw you're building Nynch, a growth platform specifically for consultants and fractional professionals. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr"/>
-      <c r="K77" s="2" t="inlineStr">
+      <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4579,11 +4965,16 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
           <t>Hey Michael, saw you discuss AI integration in podcast production at Fame. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr"/>
-      <c r="K78" s="2" t="inlineStr">
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4632,11 +5023,16 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
           <t>Hey Oyinkro, saw you're positioning K.OS VISUALS as a creative GTM partner for fast-growing AI/SaaS companies. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr"/>
-      <c r="K79" s="2" t="inlineStr">
+      <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4685,11 +5081,16 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
           <t>Hey Costin, saw you turn complex SaaS products into clear, high-impact video as a strategic video partner. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr"/>
-      <c r="K80" s="2" t="inlineStr">
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4738,11 +5139,16 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
           <t>Hey Marek, saw you help companies adopt DevOps culture through on-site workshops and consulting at pipetail.io. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr"/>
-      <c r="K81" s="2" t="inlineStr">
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4791,11 +5197,16 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
           <t>Hey Michal, saw you built a RAG platform for 15k+ users and now consult on DevOps culture and AI adoption. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr"/>
-      <c r="K82" s="2" t="inlineStr">
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4844,11 +5255,16 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
           <t>Hey Sara, saw you help founders and SMEs turn marketing spend into measurable growth through White Cloud Communications. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J83" s="2" t="inlineStr"/>
-      <c r="K83" s="2" t="inlineStr">
+      <c r="K83" s="2" t="inlineStr"/>
+      <c r="L83" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4897,11 +5313,16 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
           <t>Hey Jonny, saw you've been 3x Head of Marketing at B2B SaaS startups before going fractional. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J84" s="2" t="inlineStr"/>
-      <c r="K84" s="2" t="inlineStr">
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -4950,11 +5371,16 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
           <t>Hey Hugo, saw you wrote "Teams in Hell" and are a 1x exited founder now doing fractional growth work. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J85" s="2" t="inlineStr"/>
-      <c r="K85" s="2" t="inlineStr">
+      <c r="K85" s="2" t="inlineStr"/>
+      <c r="L85" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5003,11 +5429,16 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
           <t>Hey Marcus, saw your observation that companies buy AI licenses, announce it, and six months later only 10% of the team is actually using the tools. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J86" s="2" t="inlineStr"/>
-      <c r="K86" s="2" t="inlineStr">
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5056,11 +5487,16 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
           <t>Hey David, saw you build intelligent workflows and AI agents using tools like n8n, Make.com, and Airtable. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J87" s="2" t="inlineStr"/>
-      <c r="K87" s="2" t="inlineStr">
+      <c r="K87" s="2" t="inlineStr"/>
+      <c r="L87" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5109,11 +5545,16 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
           <t>Hey Matthew, saw you specialize in AI platform adoption and implementation at Mission AI Consulting. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J88" s="2" t="inlineStr"/>
-      <c r="K88" s="2" t="inlineStr">
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5162,11 +5603,16 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
           <t>Hey Adam, saw you've built a lean senior team at Growth Union for early-stage B2B SaaS clients like Writer and Recorded Future. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J89" s="2" t="inlineStr"/>
-      <c r="K89" s="2" t="inlineStr">
+      <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5215,11 +5661,16 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
           <t>Hey David, saw you're building Lynx Growth Agency around AI-driven marketing and automation. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J90" s="2" t="inlineStr"/>
-      <c r="K90" s="2" t="inlineStr">
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5268,11 +5719,16 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
           <t>Hey Alex, saw your writing on AI agents in RevOps as CEO of Forecastio. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J91" s="2" t="inlineStr"/>
-      <c r="K91" s="2" t="inlineStr">
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5321,11 +5777,16 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
           <t>Hey Kristofer, saw your tagline about helping startups supercharge their small RevOps teams. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr"/>
-      <c r="K92" s="2" t="inlineStr">
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5374,11 +5835,16 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
           <t>Hey Shaun, saw you're building agentic AI systems as an AI Marketing Engineer while running thisisagency.ai. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J93" s="2" t="inlineStr"/>
-      <c r="K93" s="2" t="inlineStr">
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5427,11 +5893,16 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
           <t>Hey Sam, saw you're running Origin 63 as a small, results-focused growth agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J94" s="2" t="inlineStr"/>
-      <c r="K94" s="2" t="inlineStr">
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5480,11 +5951,16 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
           <t>Hey Josh, saw your work on revenue growth and retention at Hüify, a HubSpot partner agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J95" s="2" t="inlineStr"/>
-      <c r="K95" s="2" t="inlineStr">
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5533,11 +6009,16 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
           <t>Hey Clwyd, saw you work as an AI consultant at Whitehat, helping businesses adopt AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J96" s="2" t="inlineStr"/>
-      <c r="K96" s="2" t="inlineStr">
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5586,11 +6067,16 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
           <t>Hey Clara, saw you're employee #3 and Chief of Staff at Kairos. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J97" s="2" t="inlineStr"/>
-      <c r="K97" s="2" t="inlineStr">
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5639,11 +6125,16 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
           <t>Hey Riddhi, saw you're running Thought In A Dot as a content marketing agency and brand strategist. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J98" s="2" t="inlineStr"/>
-      <c r="K98" s="2" t="inlineStr">
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5692,11 +6183,16 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
           <t>Hey John, saw you founded Creative Engine, a branding and digital marketing agency in Austin. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J99" s="2" t="inlineStr"/>
-      <c r="K99" s="2" t="inlineStr">
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5745,11 +6241,16 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
           <t>Hey Laney, saw you run The Design Boutique and pride yourselves on being able to pivot quickly as a small shop. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J100" s="2" t="inlineStr"/>
-      <c r="K100" s="2" t="inlineStr">
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5798,11 +6299,16 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
           <t>Hey Thomas, saw you founded Venture Visuals, a creative agency in Seattle. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J101" s="2" t="inlineStr"/>
-      <c r="K101" s="2" t="inlineStr">
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5851,11 +6357,16 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
           <t>Hey Santosh, saw you're running Visual Best, an AI creative production agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J102" s="2" t="inlineStr"/>
-      <c r="K102" s="2" t="inlineStr">
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5904,11 +6415,16 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
           <t>Hey David, saw you describe your business as having an AI-first mindset while running Sounds Good Agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J103" s="2" t="inlineStr"/>
-      <c r="K103" s="2" t="inlineStr">
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -5957,11 +6473,16 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
           <t>Hey Mark, saw you're a pioneer in AI-native software engineering as founder of SoftwareFactory.ai. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J104" s="2" t="inlineStr"/>
-      <c r="K104" s="2" t="inlineStr">
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6010,11 +6531,16 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
           <t>Hey Dylan, saw you install AI systems into service businesses as an independent consultant. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J105" s="2" t="inlineStr"/>
-      <c r="K105" s="2" t="inlineStr">
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6063,11 +6589,16 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
           <t>Hey Alex, saw you're co-founder/CEO of Intryc, a Y Combinator S24 startup. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J106" s="2" t="inlineStr"/>
-      <c r="K106" s="2" t="inlineStr">
+      <c r="K106" s="2" t="inlineStr"/>
+      <c r="L106" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6116,11 +6647,16 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
           <t>Hey Arham, saw you founded Pixated, a performance marketing agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J107" s="2" t="inlineStr"/>
-      <c r="K107" s="2" t="inlineStr">
+      <c r="K107" s="2" t="inlineStr"/>
+      <c r="L107" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6169,11 +6705,16 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
           <t>Hey Alex, saw you're scaling DTC ecommerce brands through Tierra. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J108" s="2" t="inlineStr"/>
-      <c r="K108" s="2" t="inlineStr">
+      <c r="K108" s="2" t="inlineStr"/>
+      <c r="L108" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6222,11 +6763,16 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
           <t>Hey Beckie, saw you run a boutique recruiting agency with a niche sector focus. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J109" s="2" t="inlineStr"/>
-      <c r="K109" s="2" t="inlineStr">
+      <c r="K109" s="2" t="inlineStr"/>
+      <c r="L109" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6275,11 +6821,16 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
           <t>Hey Katie, saw your writing on balancing technology and human connection in recruiting at CollabRecruit. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J110" s="2" t="inlineStr"/>
-      <c r="K110" s="2" t="inlineStr">
+      <c r="K110" s="2" t="inlineStr"/>
+      <c r="L110" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6328,11 +6879,16 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
           <t>Hey Jennifer, saw you founded Bookkeeping Done Right to serve small and medium businesses in South Florida. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J111" s="2" t="inlineStr"/>
-      <c r="K111" s="2" t="inlineStr">
+      <c r="K111" s="2" t="inlineStr"/>
+      <c r="L111" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6381,11 +6937,16 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
           <t>Hey Parry, saw you're leading a team of senior PR leaders at Crackle PR. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J112" s="2" t="inlineStr"/>
-      <c r="K112" s="2" t="inlineStr">
+      <c r="K112" s="2" t="inlineStr"/>
+      <c r="L112" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6434,11 +6995,16 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
           <t>Hey Carin, saw your writing on AI strategy in communications. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J113" s="2" t="inlineStr"/>
-      <c r="K113" s="2" t="inlineStr">
+      <c r="K113" s="2" t="inlineStr"/>
+      <c r="L113" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6487,11 +7053,16 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
           <t>Hey Erika, saw you're running 85th &amp; Park, a culture-driven creative marketing and comms agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J114" s="2" t="inlineStr"/>
-      <c r="K114" s="2" t="inlineStr">
+      <c r="K114" s="2" t="inlineStr"/>
+      <c r="L114" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6540,11 +7111,16 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
           <t>Hey Sam, saw you just founded a new AI automation agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J115" s="2" t="inlineStr"/>
-      <c r="K115" s="2" t="inlineStr">
+      <c r="K115" s="2" t="inlineStr"/>
+      <c r="L115" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6593,11 +7169,16 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
           <t>Hey M, saw you're running your own web design agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J116" s="2" t="inlineStr"/>
-      <c r="K116" s="2" t="inlineStr">
+      <c r="K116" s="2" t="inlineStr"/>
+      <c r="L116" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6646,11 +7227,16 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
           <t>Hey Kristen, saw your interest in AI adoption for web design and development. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J117" s="2" t="inlineStr"/>
-      <c r="K117" s="2" t="inlineStr">
+      <c r="K117" s="2" t="inlineStr"/>
+      <c r="L117" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6699,11 +7285,16 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
           <t>Hey Stefen, saw you co-founded Kelp Creative Agency. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J118" s="2" t="inlineStr"/>
-      <c r="K118" s="2" t="inlineStr">
+      <c r="K118" s="2" t="inlineStr"/>
+      <c r="L118" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6752,11 +7343,16 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
           <t>Hey Dean, saw you're co-founder and Head of Operations at Superstate. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J119" s="2" t="inlineStr"/>
-      <c r="K119" s="2" t="inlineStr">
+      <c r="K119" s="2" t="inlineStr"/>
+      <c r="L119" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6805,11 +7401,16 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
           <t>Hey Leah, saw you're co-founder and Head of Operations at See Jane Drill. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J120" s="2" t="inlineStr"/>
-      <c r="K120" s="2" t="inlineStr">
+      <c r="K120" s="2" t="inlineStr"/>
+      <c r="L120" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6858,11 +7459,16 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
           <t>Hey Evan, saw you're using AI tools like Heygen and Freepik at Boomin' Brands Media. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J121" s="2" t="inlineStr"/>
-      <c r="K121" s="2" t="inlineStr">
+      <c r="K121" s="2" t="inlineStr"/>
+      <c r="L121" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6911,11 +7517,16 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
           <t>Hey Yash, saw your AI-led creative production work at Lemonade Creatives. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J122" s="2" t="inlineStr"/>
-      <c r="K122" s="2" t="inlineStr">
+      <c r="K122" s="2" t="inlineStr"/>
+      <c r="L122" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -6964,11 +7575,16 @@
       </c>
       <c r="I123" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
           <t>Hey Adam, saw you built Taia, a workflow system addressing friction in translation processes. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J123" s="2" t="inlineStr"/>
-      <c r="K123" s="2" t="inlineStr">
+      <c r="K123" s="2" t="inlineStr"/>
+      <c r="L123" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7017,11 +7633,16 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
           <t>Hey Adriana, saw you run Libre Design Studio specifically for founders and startups. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J124" s="2" t="inlineStr"/>
-      <c r="K124" s="2" t="inlineStr">
+      <c r="K124" s="2" t="inlineStr"/>
+      <c r="L124" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7070,11 +7691,16 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
           <t>Hey Atiqur, saw you founded Design Monks. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J125" s="2" t="inlineStr"/>
-      <c r="K125" s="2" t="inlineStr">
+      <c r="K125" s="2" t="inlineStr"/>
+      <c r="L125" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7123,11 +7749,16 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
           <t>Hey Thomas, saw you help B2B SaaS companies turn Customer Success into measurable revenue at Revora Consultants. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J126" s="2" t="inlineStr"/>
-      <c r="K126" s="2" t="inlineStr">
+      <c r="K126" s="2" t="inlineStr"/>
+      <c r="L126" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7176,11 +7807,16 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
           <t>Hey Peter, saw you're building Trendin, an AI-native operating system for influencer agencies. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J127" s="2" t="inlineStr"/>
-      <c r="K127" s="2" t="inlineStr">
+      <c r="K127" s="2" t="inlineStr"/>
+      <c r="L127" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7229,11 +7865,16 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
           <t>Hey Krishna, saw you built LegalConnect to deliver AI-drafted, solicitor-reviewed legal documents for SMEs. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J128" s="2" t="inlineStr"/>
-      <c r="K128" s="2" t="inlineStr">
+      <c r="K128" s="2" t="inlineStr"/>
+      <c r="L128" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7282,11 +7923,16 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
           <t>Hey Jay, saw you run Startup Legal Group, serving startup clients directly. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J129" s="2" t="inlineStr"/>
-      <c r="K129" s="2" t="inlineStr">
+      <c r="K129" s="2" t="inlineStr"/>
+      <c r="L129" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7335,11 +7981,16 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
           <t>Hey Nahme, saw you're running Research Connections, a market research consulting and field management company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J130" s="2" t="inlineStr"/>
-      <c r="K130" s="2" t="inlineStr">
+      <c r="K130" s="2" t="inlineStr"/>
+      <c r="L130" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7388,11 +8039,16 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
           <t>Hey Jake, saw you run JakeWu Market Research, a small solo-founder shop. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J131" s="2" t="inlineStr"/>
-      <c r="K131" s="2" t="inlineStr">
+      <c r="K131" s="2" t="inlineStr"/>
+      <c r="L131" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7441,11 +8097,16 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
           <t>Hey Jenna, saw you founded an education platform teaching interior designers to use AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J132" s="2" t="inlineStr"/>
-      <c r="K132" s="2" t="inlineStr">
+      <c r="K132" s="2" t="inlineStr"/>
+      <c r="L132" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7494,11 +8155,16 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
           <t>Hey Nina, saw you co-founded Curioso, an assemblage of designers, architects, and business-minded creatives. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J133" s="2" t="inlineStr"/>
-      <c r="K133" s="2" t="inlineStr">
+      <c r="K133" s="2" t="inlineStr"/>
+      <c r="L133" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7547,11 +8213,16 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
           <t>Hey Snehadeep, saw you use AI-driven design tools as founder of Studio ORCHIVIZ. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J134" s="2" t="inlineStr"/>
-      <c r="K134" s="2" t="inlineStr">
+      <c r="K134" s="2" t="inlineStr"/>
+      <c r="L134" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7600,11 +8271,16 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
           <t>Hey Akeem, saw you're co-founder of Thread, a YC W23 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J135" s="2" t="inlineStr"/>
-      <c r="K135" s="2" t="inlineStr">
+      <c r="K135" s="2" t="inlineStr"/>
+      <c r="L135" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7653,11 +8329,16 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
           <t>Hey Ty, saw you're co-founder and CEO of inBuild, a YC W23 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J136" s="2" t="inlineStr"/>
-      <c r="K136" s="2" t="inlineStr">
+      <c r="K136" s="2" t="inlineStr"/>
+      <c r="L136" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7706,11 +8387,16 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
           <t>Hey Vlad, saw you're co-founder of Infisical, a YC W23 company. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J137" s="2" t="inlineStr"/>
-      <c r="K137" s="2" t="inlineStr">
+      <c r="K137" s="2" t="inlineStr"/>
+      <c r="L137" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7759,11 +8445,16 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
           <t>Hey Neel, saw you're co-founder of Clueso, an AI video creation company from YC W23. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J138" s="2" t="inlineStr"/>
-      <c r="K138" s="2" t="inlineStr">
+      <c r="K138" s="2" t="inlineStr"/>
+      <c r="L138" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7812,11 +8503,16 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
           <t>Hey Sourav, saw you focus on brand strategy specifically for early-stage startups at Branded Minds. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J139" s="2" t="inlineStr"/>
-      <c r="K139" s="2" t="inlineStr">
+      <c r="K139" s="2" t="inlineStr"/>
+      <c r="L139" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7865,11 +8561,16 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
           <t>Hey Ulli, saw you run First The Trousers as a brand strategy and positioning consultancy. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J140" s="2" t="inlineStr"/>
-      <c r="K140" s="2" t="inlineStr">
+      <c r="K140" s="2" t="inlineStr"/>
+      <c r="L140" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7918,11 +8619,16 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
           <t>Hey Lance, saw you're building BrandChef.ai. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J141" s="2" t="inlineStr"/>
-      <c r="K141" s="2" t="inlineStr">
+      <c r="K141" s="2" t="inlineStr"/>
+      <c r="L141" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -7971,11 +8677,16 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
           <t>Hey Branden, saw you founded Build, a branding agency built around practical design. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J142" s="2" t="inlineStr"/>
-      <c r="K142" s="2" t="inlineStr">
+      <c r="K142" s="2" t="inlineStr"/>
+      <c r="L142" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8024,11 +8735,16 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
           <t>Hey Jill, saw you run Your HR Partners as a boutique human resources services company. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J143" s="2" t="inlineStr"/>
-      <c r="K143" s="2" t="inlineStr">
+      <c r="K143" s="2" t="inlineStr"/>
+      <c r="L143" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8077,11 +8793,16 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
           <t>Hey Apoorv, saw you're helping B2B SaaS companies with AI search visibility at Found On AI. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J144" s="2" t="inlineStr"/>
-      <c r="K144" s="2" t="inlineStr">
+      <c r="K144" s="2" t="inlineStr"/>
+      <c r="L144" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8130,11 +8851,16 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
           <t>Hey Matt, saw you co-founded Sheepdog Projects to offer BI consulting and data strategy services. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J145" s="2" t="inlineStr"/>
-      <c r="K145" s="2" t="inlineStr">
+      <c r="K145" s="2" t="inlineStr"/>
+      <c r="L145" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8183,11 +8909,16 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
           <t>Hey Jason, saw you discuss how AI is being integrated into podcast production workflows at B2B Better. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J146" s="2" t="inlineStr"/>
-      <c r="K146" s="2" t="inlineStr">
+      <c r="K146" s="2" t="inlineStr"/>
+      <c r="L146" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8236,11 +8967,16 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
           <t>Hey Samuel, saw you run a fractional CMO agency in New York. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J147" s="2" t="inlineStr"/>
-      <c r="K147" s="2" t="inlineStr">
+      <c r="K147" s="2" t="inlineStr"/>
+      <c r="L147" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8289,11 +9025,16 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
           <t>Hey Joshua, saw you're driving data-driven growth for clients as founder of sōsh. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J148" s="2" t="inlineStr"/>
-      <c r="K148" s="2" t="inlineStr">
+      <c r="K148" s="2" t="inlineStr"/>
+      <c r="L148" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8342,11 +9083,16 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
+          <t>Question about your team and AI tools</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
           <t>Hey Kristen, saw you co-founded a boutique full-service digital marketing consulting firm for B2B professional services. Question for you: does your team use ChatGPT or Claude much, and if so, is it mostly everyone working solo, or is there any shared visibility into what people are trying or deciding? Curious how you all handle it.</t>
         </is>
       </c>
-      <c r="J149" s="2" t="inlineStr"/>
-      <c r="K149" s="2" t="inlineStr">
+      <c r="K149" s="2" t="inlineStr"/>
+      <c r="L149" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8395,11 +9141,16 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
           <t>Hey Dawn, saw you partner with early-stage founders and CEOs to build brands that scale. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J150" s="2" t="inlineStr"/>
-      <c r="K150" s="2" t="inlineStr">
+      <c r="K150" s="2" t="inlineStr"/>
+      <c r="L150" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8448,11 +9199,16 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
+          <t>Question about your clients and AI tools</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
           <t>Hey Miranda, saw you're empowering small businesses with AI tools and services through AI Consulting Network. Question for you: across the teams or clients you work with, is AI tool usage mostly a solo thing per person, or is there any shared visibility into what's being tried? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J151" s="2" t="inlineStr"/>
-      <c r="K151" s="2" t="inlineStr">
+      <c r="K151" s="2" t="inlineStr"/>
+      <c r="L151" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8460,7 +9216,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8626,7 +9382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8637,9 +9393,10 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="65" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8685,15 +9442,20 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Draft Message</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Date Found</t>
         </is>
@@ -8742,11 +9504,16 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>Question about AI usage in your community</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Hey Darrell, saw your newsletter on marketing ops team structure and career growth. Question for you: is solo AI tool usage with little shared visibility across a team something you hear about often from your community? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8795,11 +9562,16 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
+          <t>Question about AI usage in your community</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>Hey Jen, saw your weekly newsletter for the marketing ops community. Question for you: is solo AI tool usage with little shared visibility across a team something you hear about often from your community? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8848,11 +9620,16 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
+          <t>Question about AI usage in your community</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>Hey Mike, saw MO Pros hitting 4,000+ marketing/RevOps members. Question for you: is solo AI tool usage with little shared visibility across a team something you hear about often from your community? Curious what you're seeing.</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
@@ -8860,7 +9637,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approved,Rejected"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>